<commit_message>
Adding more test field in harshit page of wikipedia-Testing-ExcelSheet.xlsx
</commit_message>
<xml_diff>
--- a/wikipedia-Testing-ExcelSheet.xlsx
+++ b/wikipedia-Testing-ExcelSheet.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\PROJECT\wikipedia_testing\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\PROJECT\Wikipedia_testing_maben\wikipedia_testing_Maven\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4CFD59CC-5CD2-4CA8-823B-2BBD480A652A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BF22E6B2-3DAC-4B9E-B61A-D22C47808603}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="11424" yWindow="0" windowWidth="11712" windowHeight="13776" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Akash" sheetId="1" r:id="rId1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="155" uniqueCount="86">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="211" uniqueCount="116">
   <si>
     <t>Wikipedia Search &amp; Reader UI</t>
   </si>
@@ -324,15 +324,6 @@
     <t>Test status(Pass/Fail)</t>
   </si>
   <si>
-    <t>valid_Keyword</t>
-  </si>
-  <si>
-    <t>sdgfgsi</t>
-  </si>
-  <si>
-    <t>giuis</t>
-  </si>
-  <si>
     <r>
       <rPr>
         <sz val="12"/>
@@ -467,12 +458,111 @@
   <si>
     <t>Scroll from top to bottom of article</t>
   </si>
+  <si>
+    <t>valid_Keyword_India</t>
+  </si>
+  <si>
+    <t>search</t>
+  </si>
+  <si>
+    <t>valid keyword search</t>
+  </si>
+  <si>
+    <t>india</t>
+  </si>
+  <si>
+    <t>none</t>
+  </si>
+  <si>
+    <t>Valid_keyword_Java</t>
+  </si>
+  <si>
+    <t>Another valid keyword</t>
+  </si>
+  <si>
+    <t>java</t>
+  </si>
+  <si>
+    <t>Invalid_keyword</t>
+  </si>
+  <si>
+    <t>Invalid keyword search</t>
+  </si>
+  <si>
+    <t>xyzabc123</t>
+  </si>
+  <si>
+    <t>Empty_search</t>
+  </si>
+  <si>
+    <t>Empty search validation</t>
+  </si>
+  <si>
+    <t>empty</t>
+  </si>
+  <si>
+    <t>Numbers</t>
+  </si>
+  <si>
+    <t>Numeric input</t>
+  </si>
+  <si>
+    <t>Special_characters</t>
+  </si>
+  <si>
+    <t>Special-character input</t>
+  </si>
+  <si>
+    <t>@#$%^&amp;*</t>
+  </si>
+  <si>
+    <t>Long_search_text</t>
+  </si>
+  <si>
+    <t>seach</t>
+  </si>
+  <si>
+    <t>Long input validation</t>
+  </si>
+  <si>
+    <t>Long text</t>
+  </si>
+  <si>
+    <t>Search_suggestions</t>
+  </si>
+  <si>
+    <t>Search Suggestions</t>
+  </si>
+  <si>
+    <t>Verify suggestions</t>
+  </si>
+  <si>
+    <t>ind</t>
+  </si>
+  <si>
+    <t>Search_results_verification</t>
+  </si>
+  <si>
+    <t>search results</t>
+  </si>
+  <si>
+    <t>Verify correct results</t>
+  </si>
+  <si>
+    <t>Search_result_se_article_open_hona</t>
+  </si>
+  <si>
+    <t>Article Reader</t>
+  </si>
+  <si>
+    <t>Verify article opens</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="8">
+  <fonts count="9">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -533,6 +623,11 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="14"/>
+      <color theme="1"/>
+      <name val="Arial Unicode MS"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -554,7 +649,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="21">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -610,6 +705,9 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -991,7 +1089,7 @@
         <v>12</v>
       </c>
       <c r="C7" s="7" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
       <c r="D7" s="4" t="s">
         <v>13</v>
@@ -1017,7 +1115,7 @@
         <v>18</v>
       </c>
       <c r="C8" s="7" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
       <c r="D8" s="4" t="s">
         <v>19</v>
@@ -1069,7 +1167,7 @@
         <v>27</v>
       </c>
       <c r="C10" s="7" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
       <c r="D10" s="4" t="s">
         <v>28</v>
@@ -1095,7 +1193,7 @@
         <v>32</v>
       </c>
       <c r="C11" s="7" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
       <c r="D11" s="4" t="s">
         <v>33</v>
@@ -1121,7 +1219,7 @@
         <v>36</v>
       </c>
       <c r="C12" s="7" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
       <c r="D12" s="4" t="s">
         <v>37</v>
@@ -1147,7 +1245,7 @@
         <v>40</v>
       </c>
       <c r="C13" s="7" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
       <c r="D13" s="4" t="s">
         <v>41</v>
@@ -1173,7 +1271,7 @@
         <v>44</v>
       </c>
       <c r="C14" s="7" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
       <c r="D14" s="4" t="s">
         <v>45</v>
@@ -1199,7 +1297,7 @@
         <v>48</v>
       </c>
       <c r="C15" s="7" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
       <c r="D15" s="4" t="s">
         <v>49</v>
@@ -1225,7 +1323,7 @@
         <v>52</v>
       </c>
       <c r="C16" s="7" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
       <c r="D16" s="7" t="s">
         <v>53</v>
@@ -1248,22 +1346,22 @@
         <v>11</v>
       </c>
       <c r="B17" s="7" t="s">
+        <v>61</v>
+      </c>
+      <c r="C17" s="7" t="s">
+        <v>75</v>
+      </c>
+      <c r="D17" s="7" t="s">
+        <v>62</v>
+      </c>
+      <c r="E17" s="7" t="s">
+        <v>63</v>
+      </c>
+      <c r="F17" s="8" t="s">
+        <v>65</v>
+      </c>
+      <c r="G17" s="7" t="s">
         <v>64</v>
-      </c>
-      <c r="C17" s="7" t="s">
-        <v>78</v>
-      </c>
-      <c r="D17" s="7" t="s">
-        <v>65</v>
-      </c>
-      <c r="E17" s="7" t="s">
-        <v>66</v>
-      </c>
-      <c r="F17" s="8" t="s">
-        <v>68</v>
-      </c>
-      <c r="G17" s="7" t="s">
-        <v>67</v>
       </c>
       <c r="H17" s="4" t="s">
         <v>17</v>
@@ -1274,19 +1372,19 @@
         <v>12</v>
       </c>
       <c r="B18" s="7" t="s">
+        <v>66</v>
+      </c>
+      <c r="C18" s="7" t="s">
+        <v>75</v>
+      </c>
+      <c r="D18" s="7" t="s">
+        <v>67</v>
+      </c>
+      <c r="E18" s="7" t="s">
+        <v>68</v>
+      </c>
+      <c r="F18" s="8" t="s">
         <v>69</v>
-      </c>
-      <c r="C18" s="7" t="s">
-        <v>78</v>
-      </c>
-      <c r="D18" s="7" t="s">
-        <v>70</v>
-      </c>
-      <c r="E18" s="7" t="s">
-        <v>71</v>
-      </c>
-      <c r="F18" s="8" t="s">
-        <v>72</v>
       </c>
       <c r="G18" s="7" t="s">
         <v>16</v>
@@ -1300,19 +1398,19 @@
         <v>13</v>
       </c>
       <c r="B19" s="7" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="C19" s="7" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
       <c r="D19" s="7" t="s">
-        <v>73</v>
+        <v>70</v>
       </c>
       <c r="E19" s="7" t="s">
-        <v>74</v>
+        <v>71</v>
       </c>
       <c r="F19" s="8" t="s">
-        <v>75</v>
+        <v>72</v>
       </c>
       <c r="G19" s="7" t="s">
         <v>16</v>
@@ -1326,19 +1424,19 @@
         <v>14</v>
       </c>
       <c r="B20" s="7" t="s">
+        <v>76</v>
+      </c>
+      <c r="C20" s="7" t="s">
+        <v>75</v>
+      </c>
+      <c r="D20" s="7" t="s">
+        <v>77</v>
+      </c>
+      <c r="E20" s="7" t="s">
+        <v>78</v>
+      </c>
+      <c r="F20" s="8" t="s">
         <v>79</v>
-      </c>
-      <c r="C20" s="7" t="s">
-        <v>78</v>
-      </c>
-      <c r="D20" s="7" t="s">
-        <v>80</v>
-      </c>
-      <c r="E20" s="7" t="s">
-        <v>81</v>
-      </c>
-      <c r="F20" s="8" t="s">
-        <v>82</v>
       </c>
       <c r="G20" s="7" t="s">
         <v>16</v>
@@ -1352,16 +1450,16 @@
         <v>15</v>
       </c>
       <c r="B21" s="7" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="C21" s="7" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
       <c r="D21" s="7" t="s">
-        <v>84</v>
+        <v>81</v>
       </c>
       <c r="E21" s="7" t="s">
-        <v>85</v>
+        <v>82</v>
       </c>
       <c r="F21" s="8"/>
       <c r="G21" s="7" t="s">
@@ -2485,7 +2583,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:H10"/>
+  <dimension ref="A1:H16"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.4"/>
   <cols>
     <col min="1" max="1" width="14.6640625" customWidth="1"/>
@@ -2583,22 +2681,245 @@
       </c>
     </row>
     <row r="7" spans="1:8" ht="128.4" customHeight="1">
-      <c r="A7">
+      <c r="A7" s="7">
         <v>1</v>
       </c>
-      <c r="B7" t="s">
-        <v>58</v>
-      </c>
-      <c r="C7" t="s">
-        <v>59</v>
-      </c>
-      <c r="D7" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="8" spans="1:8" ht="117.6" customHeight="1"/>
-    <row r="9" spans="1:8" ht="88.8" customHeight="1"/>
-    <row r="10" spans="1:8" ht="109.8" customHeight="1"/>
+      <c r="B7" s="7" t="s">
+        <v>83</v>
+      </c>
+      <c r="C7" s="7" t="s">
+        <v>84</v>
+      </c>
+      <c r="D7" s="7" t="s">
+        <v>85</v>
+      </c>
+      <c r="E7" s="7" t="s">
+        <v>86</v>
+      </c>
+      <c r="F7" s="7"/>
+      <c r="G7" s="7" t="s">
+        <v>64</v>
+      </c>
+      <c r="H7" s="7" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" ht="117.6" customHeight="1">
+      <c r="A8" s="7">
+        <v>2</v>
+      </c>
+      <c r="B8" s="7" t="s">
+        <v>88</v>
+      </c>
+      <c r="C8" s="7" t="s">
+        <v>84</v>
+      </c>
+      <c r="D8" s="7" t="s">
+        <v>89</v>
+      </c>
+      <c r="E8" s="7" t="s">
+        <v>90</v>
+      </c>
+      <c r="F8" s="7"/>
+      <c r="G8" s="7" t="s">
+        <v>64</v>
+      </c>
+      <c r="H8" s="7" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" ht="88.8" customHeight="1">
+      <c r="A9" s="7">
+        <v>3</v>
+      </c>
+      <c r="B9" s="7" t="s">
+        <v>91</v>
+      </c>
+      <c r="C9" s="7" t="s">
+        <v>84</v>
+      </c>
+      <c r="D9" s="7" t="s">
+        <v>92</v>
+      </c>
+      <c r="E9" s="7" t="s">
+        <v>93</v>
+      </c>
+      <c r="F9" s="7"/>
+      <c r="G9" s="7" t="s">
+        <v>64</v>
+      </c>
+      <c r="H9" s="7" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" ht="109.8" customHeight="1">
+      <c r="A10" s="7">
+        <v>4</v>
+      </c>
+      <c r="B10" s="7" t="s">
+        <v>94</v>
+      </c>
+      <c r="C10" s="7" t="s">
+        <v>84</v>
+      </c>
+      <c r="D10" s="7" t="s">
+        <v>95</v>
+      </c>
+      <c r="E10" s="7" t="s">
+        <v>96</v>
+      </c>
+      <c r="F10" s="7"/>
+      <c r="G10" s="7" t="s">
+        <v>64</v>
+      </c>
+      <c r="H10" s="7" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8" ht="18">
+      <c r="A11" s="7">
+        <v>5</v>
+      </c>
+      <c r="B11" s="7" t="s">
+        <v>97</v>
+      </c>
+      <c r="C11" s="7" t="s">
+        <v>84</v>
+      </c>
+      <c r="D11" s="7" t="s">
+        <v>98</v>
+      </c>
+      <c r="E11" s="7">
+        <v>123456</v>
+      </c>
+      <c r="F11" s="7"/>
+      <c r="G11" s="7" t="s">
+        <v>64</v>
+      </c>
+      <c r="H11" s="7" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8" ht="36">
+      <c r="A12" s="7">
+        <v>6</v>
+      </c>
+      <c r="B12" s="7" t="s">
+        <v>99</v>
+      </c>
+      <c r="C12" s="7" t="s">
+        <v>84</v>
+      </c>
+      <c r="D12" s="7" t="s">
+        <v>100</v>
+      </c>
+      <c r="E12" s="20" t="s">
+        <v>101</v>
+      </c>
+      <c r="F12" s="7"/>
+      <c r="G12" s="7" t="s">
+        <v>64</v>
+      </c>
+      <c r="H12" s="7" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8" ht="18">
+      <c r="A13" s="7">
+        <v>7</v>
+      </c>
+      <c r="B13" s="7" t="s">
+        <v>102</v>
+      </c>
+      <c r="C13" s="7" t="s">
+        <v>103</v>
+      </c>
+      <c r="D13" s="7" t="s">
+        <v>104</v>
+      </c>
+      <c r="E13" s="7" t="s">
+        <v>105</v>
+      </c>
+      <c r="F13" s="7"/>
+      <c r="G13" s="7" t="s">
+        <v>64</v>
+      </c>
+      <c r="H13" s="7" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="14" spans="1:8" ht="36">
+      <c r="A14" s="7">
+        <v>8</v>
+      </c>
+      <c r="B14" s="7" t="s">
+        <v>106</v>
+      </c>
+      <c r="C14" s="7" t="s">
+        <v>107</v>
+      </c>
+      <c r="D14" s="7" t="s">
+        <v>108</v>
+      </c>
+      <c r="E14" s="7" t="s">
+        <v>109</v>
+      </c>
+      <c r="F14" s="7"/>
+      <c r="G14" s="7" t="s">
+        <v>64</v>
+      </c>
+      <c r="H14" s="7" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="15" spans="1:8" ht="36">
+      <c r="A15" s="7">
+        <v>9</v>
+      </c>
+      <c r="B15" s="7" t="s">
+        <v>110</v>
+      </c>
+      <c r="C15" s="7" t="s">
+        <v>111</v>
+      </c>
+      <c r="D15" s="7" t="s">
+        <v>112</v>
+      </c>
+      <c r="E15" s="7" t="s">
+        <v>86</v>
+      </c>
+      <c r="F15" s="7"/>
+      <c r="G15" s="7" t="s">
+        <v>64</v>
+      </c>
+      <c r="H15" s="7" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="16" spans="1:8" ht="54">
+      <c r="A16" s="7">
+        <v>10</v>
+      </c>
+      <c r="B16" s="7" t="s">
+        <v>113</v>
+      </c>
+      <c r="C16" s="7" t="s">
+        <v>114</v>
+      </c>
+      <c r="D16" s="7" t="s">
+        <v>115</v>
+      </c>
+      <c r="E16" s="7" t="s">
+        <v>86</v>
+      </c>
+      <c r="F16" s="7"/>
+      <c r="G16" s="7" t="s">
+        <v>64</v>
+      </c>
+      <c r="H16" s="7" t="s">
+        <v>87</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="4">
     <mergeCell ref="A1:H3"/>
@@ -2667,7 +2988,7 @@
       <c r="D4" s="17"/>
       <c r="E4" s="17"/>
       <c r="F4" s="17" t="s">
-        <v>61</v>
+        <v>58</v>
       </c>
       <c r="G4" s="17"/>
       <c r="H4" s="17"/>
@@ -2702,10 +3023,10 @@
         <v>9</v>
       </c>
       <c r="G6" s="1" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="H6" s="1" t="s">
-        <v>63</v>
+        <v>60</v>
       </c>
     </row>
   </sheetData>
@@ -2777,7 +3098,7 @@
       <c r="D4" s="17"/>
       <c r="E4" s="17"/>
       <c r="F4" s="17" t="s">
-        <v>61</v>
+        <v>58</v>
       </c>
       <c r="G4" s="17"/>
       <c r="H4" s="17"/>
@@ -2812,10 +3133,10 @@
         <v>9</v>
       </c>
       <c r="G6" s="1" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="H6" s="1" t="s">
-        <v>63</v>
+        <v>60</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
adding new test cases in excel file 'WIKIPEDIA-Testing-Excelsheet' by lucky sharma
</commit_message>
<xml_diff>
--- a/wikipedia-Testing-ExcelSheet.xlsx
+++ b/wikipedia-Testing-ExcelSheet.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30430"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="27726"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\PROJECT\Wikipedia_testing_maben\wikipedia_testing_Maven\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\CRC_5th_Devops_182\wikipedia_testing_Maven\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BF22E6B2-3DAC-4B9E-B61A-D22C47808603}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FFFEE222-86C5-46A6-AF9B-DF9DB543D35F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Akash" sheetId="1" r:id="rId1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="211" uniqueCount="116">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="379" uniqueCount="195">
   <si>
     <t>Wikipedia Search &amp; Reader UI</t>
   </si>
@@ -556,6 +556,348 @@
   </si>
   <si>
     <t>Verify article opens</t>
+  </si>
+  <si>
+    <t>working</t>
+  </si>
+  <si>
+    <t>N/A</t>
+  </si>
+  <si>
+    <t>BUG/ISSUE</t>
+  </si>
+  <si>
+    <t>Language_Search_Test.java</t>
+  </si>
+  <si>
+    <t>Language Testing</t>
+  </si>
+  <si>
+    <t>Check Hindi language search from language dropdown</t>
+  </si>
+  <si>
+    <t>Select Hindi from dropdown and search 'भारत'</t>
+  </si>
+  <si>
+    <t>1. Open ChromeBrowser
+2. Go to Wikipedia (https://www.wikipedia.org)
+3. Select 'Hindi' from the language dropdown
+4. Enter 'भारत' in search box
+5. Click on Search button
+6. Check URL contains 'hi.wikipedia.org' and article page is displayed in Hindi</t>
+  </si>
+  <si>
+    <t>Check English language search from language dropdown</t>
+  </si>
+  <si>
+    <t>Select English from dropdown and search 'India'</t>
+  </si>
+  <si>
+    <t>1. Open ChromeBrowser
+2. Go to Wikipedia (https://www.wikipedia.org)
+3. Select 'English' from the language dropdown
+4. Enter 'India' in search box
+5. Click on Search button
+6. Check URL contains 'en.wikipedia.org' and article page is displayed in English</t>
+  </si>
+  <si>
+    <t>Check French language search from language dropdown</t>
+  </si>
+  <si>
+    <t>Select French from dropdown and search 'Inde'</t>
+  </si>
+  <si>
+    <t>1. Open ChromeBrowser
+2. Go to Wikipedia (https://www.wikipedia.org)
+3. Select 'French' from the language dropdown
+4. Enter 'Inde' in search box
+5. Click on Search button
+6. Check URL contains 'fr.wikipedia.org' and article page is displayed in French</t>
+  </si>
+  <si>
+    <t>Check German language search from language dropdown</t>
+  </si>
+  <si>
+    <t>Select German from dropdown and search 'Indien'</t>
+  </si>
+  <si>
+    <t>1. Open ChromeBrowser
+2. Go to Wikipedia (https://www.wikipedia.org)
+3. Select 'German' from the language dropdown
+4. Enter 'Indien' in search box
+5. Click on Search button
+6. Check URL contains 'de.wikipedia.org' and article page is displayed in German</t>
+  </si>
+  <si>
+    <t>Check Spanish language search from language dropdown</t>
+  </si>
+  <si>
+    <t>Select Spanish from dropdown and search 'India'</t>
+  </si>
+  <si>
+    <t>1. Open ChromeBrowser
+2. Go to Wikipedia (https://www.wikipedia.org)
+3. Select 'Spanish' from the language dropdown
+4. Enter 'India' in search box
+5. Click on Search button
+6. Check URL contains 'es.wikipedia.org' and article page is displayed in Spanish</t>
+  </si>
+  <si>
+    <t>Check Japanese language search from language dropdown</t>
+  </si>
+  <si>
+    <t>Select Japanese from dropdown and search 'インド'</t>
+  </si>
+  <si>
+    <t>1. Open ChromeBrowser
+2. Go to Wikipedia (https://www.wikipedia.org)
+3. Select 'Japanese' from the language dropdown
+4. Enter 'インド' in search box
+5. Click on Search button
+6. Check URL contains 'ja.wikipedia.org' and article page is displayed in Japanese</t>
+  </si>
+  <si>
+    <t>Check Chinese language search from language dropdown</t>
+  </si>
+  <si>
+    <t>Select Chinese from dropdown and search '印度'</t>
+  </si>
+  <si>
+    <t>1. Open ChromeBrowser
+2. Go to Wikipedia (https://www.wikipedia.org)
+3. Select 'Chinese' from the language dropdown
+4. Enter '印度' in search box
+5. Click on Search button
+6. Check URL contains 'zh.wikipedia.org' and article page is displayed in Chinese</t>
+  </si>
+  <si>
+    <t>Check Russian language search from language dropdown</t>
+  </si>
+  <si>
+    <t>Select Russian from dropdown and search 'Индия'</t>
+  </si>
+  <si>
+    <t>1. Open ChromeBrowser
+2. Go to Wikipedia (https://www.wikipedia.org)
+3. Select 'Russian' from the language dropdown
+4. Enter 'Индия' in search box
+5. Click on Search button
+6. Check URL contains 'ru.wikipedia.org' and article page is displayed in Russian</t>
+  </si>
+  <si>
+    <t>Check Arabic language search from language dropdown</t>
+  </si>
+  <si>
+    <t>Select Arabic from dropdown and search 'الهند'</t>
+  </si>
+  <si>
+    <t>1. Open ChromeBrowser
+2. Go to Wikipedia (https://www.wikipedia.org)
+3. Select 'Arabic' from the language dropdown
+4. Enter 'الهند' in search box
+5. Click on Search button
+6. Check URL contains 'ar.wikipedia.org' and article page is displayed in Arabic</t>
+  </si>
+  <si>
+    <t>Check Portuguese language search from language dropdown</t>
+  </si>
+  <si>
+    <t>Select Portuguese from dropdown and search 'Índia'</t>
+  </si>
+  <si>
+    <t>1. Open ChromeBrowser
+2. Go to Wikipedia (https://www.wikipedia.org)
+3. Select 'Portuguese' from the language dropdown
+4. Enter 'Índia' in search box
+5. Click on Search button
+6. Check URL contains 'pt.wikipedia.org' and article page is displayed in Portuguese</t>
+  </si>
+  <si>
+    <t>Check Italian language search from language dropdown</t>
+  </si>
+  <si>
+    <t>Select Italian from dropdown and search 'Italia'</t>
+  </si>
+  <si>
+    <t>1. Open ChromeBrowser
+2. Go to Wikipedia (https://www.wikipedia.org)
+3. Select 'Italian' from the language dropdown
+4. Enter 'Italia' in search box
+5. Click on Search button
+6. Check URL contains 'it.wikipedia.org' and article page is displayed in Italian</t>
+  </si>
+  <si>
+    <t>Check Korean language search from language dropdown</t>
+  </si>
+  <si>
+    <t>Select Korean from dropdown and search '인도'</t>
+  </si>
+  <si>
+    <t>1. Open ChromeBrowser
+2. Go to Wikipedia (https://www.wikipedia.org)
+3. Select 'Korean' from the language dropdown
+4. Enter '인도' in search box
+5. Click on Search button
+6. Check URL contains 'ko.wikipedia.org' and article page is displayed in Korean</t>
+  </si>
+  <si>
+    <t>Check Bengali language search from language dropdown</t>
+  </si>
+  <si>
+    <t>Select Bengali from dropdown and search 'ভারত'</t>
+  </si>
+  <si>
+    <t>1. Open ChromeBrowser
+2. Go to Wikipedia (https://www.wikipedia.org)
+3. Select 'Bengali' from the language dropdown
+4. Enter 'ভারত' in search box
+5. Click on Search button
+6. Check URL contains 'bn.wikipedia.org' and article page is displayed in Bengali</t>
+  </si>
+  <si>
+    <t>Check Tamil language search from language dropdown</t>
+  </si>
+  <si>
+    <t>Select Tamil from dropdown and search 'இந்தியா'</t>
+  </si>
+  <si>
+    <t>1. Open ChromeBrowser
+2. Go to Wikipedia (https://www.wikipedia.org)
+3. Select 'Tamil' from the language dropdown
+4. Enter 'இந்தியா' in search box
+5. Click on Search button
+6. Check URL contains 'ta.wikipedia.org' and article page is displayed in Tamil</t>
+  </si>
+  <si>
+    <t>Check Urdu language search from language dropdown</t>
+  </si>
+  <si>
+    <t>Select Urdu from dropdown and search 'بھارت'</t>
+  </si>
+  <si>
+    <t>1. Open ChromeBrowser
+2. Go to Wikipedia (https://www.wikipedia.org)
+3. Select 'Urdu' from the language dropdown
+4. Enter 'بھارت' in search box
+5. Click on Search button
+6. Check URL contains 'ur.wikipedia.org' and article page is displayed in Urdu</t>
+  </si>
+  <si>
+    <t>Language_Link_Test.java</t>
+  </si>
+  <si>
+    <t>Check Japanese language link on homepage</t>
+  </si>
+  <si>
+    <t>Click Japanese language link around the globe logo</t>
+  </si>
+  <si>
+    <t>1. Open ChromeBrowser
+2. Go to Wikipedia (https://www.wikipedia.org)
+3. Click on the Japanese link near the globe logo
+4. Check ja.wikipedia.org main page opens in Japanese</t>
+  </si>
+  <si>
+    <t>Check German language link on homepage</t>
+  </si>
+  <si>
+    <t>Click German language link around the globe logo</t>
+  </si>
+  <si>
+    <t>1. Open ChromeBrowser
+2. Go to Wikipedia (https://www.wikipedia.org)
+3. Click on the German link near the globe logo
+4. Check de.wikipedia.org main page opens in German</t>
+  </si>
+  <si>
+    <t>Check French language link on homepage</t>
+  </si>
+  <si>
+    <t>Click French language link around the globe logo</t>
+  </si>
+  <si>
+    <t>1. Open ChromeBrowser
+2. Go to Wikipedia (https://www.wikipedia.org)
+3. Click on the French link near the globe logo
+4. Check fr.wikipedia.org main page opens in French</t>
+  </si>
+  <si>
+    <t>Check Spanish language link on homepage</t>
+  </si>
+  <si>
+    <t>Click Spanish language link around the globe logo</t>
+  </si>
+  <si>
+    <t>1. Open ChromeBrowser
+2. Go to Wikipedia (https://www.wikipedia.org)
+3. Click on the Spanish link near the globe logo
+4. Check es.wikipedia.org main page opens in Spanish</t>
+  </si>
+  <si>
+    <t>Check Chinese language link on homepage</t>
+  </si>
+  <si>
+    <t>Click Chinese language link around the globe logo</t>
+  </si>
+  <si>
+    <t>1. Open ChromeBrowser
+2. Go to Wikipedia (https://www.wikipedia.org)
+3. Click on the Chinese link near the globe logo
+4. Check zh.wikipedia.org main page opens in Chinese</t>
+  </si>
+  <si>
+    <t>Check Russian language link on homepage</t>
+  </si>
+  <si>
+    <t>Click Russian language link around the globe logo</t>
+  </si>
+  <si>
+    <t>1. Open ChromeBrowser
+2. Go to Wikipedia (https://www.wikipedia.org)
+3. Click on the Russian link near the globe logo
+4. Check ru.wikipedia.org main page opens in Russian</t>
+  </si>
+  <si>
+    <t>Check Italian language link on homepage</t>
+  </si>
+  <si>
+    <t>Click Italian language link around the globe logo</t>
+  </si>
+  <si>
+    <t>1. Open ChromeBrowser
+2. Go to Wikipedia (https://www.wikipedia.org)
+3. Click on the Italian link near the globe logo
+4. Check it.wikipedia.org main page opens in Italian</t>
+  </si>
+  <si>
+    <t>Check Portuguese language link on homepage</t>
+  </si>
+  <si>
+    <t>Click Portuguese language link around the globe logo</t>
+  </si>
+  <si>
+    <t>1. Open ChromeBrowser
+2. Go to Wikipedia (https://www.wikipedia.org)
+3. Click on the Portuguese link near the globe logo
+4. Check pt.wikipedia.org main page opens in Portuguese</t>
+  </si>
+  <si>
+    <t>language_after_search.java</t>
+  </si>
+  <si>
+    <t>Check language change after searching an article</t>
+  </si>
+  <si>
+    <t>Search India, then change language from the article's Languages sidebar to Hindi</t>
+  </si>
+  <si>
+    <t>1. Open ChromeBrowser
+2. Go to Wikipedia (https://www.wikipedia.org)
+3. Search India
+4. Click on Search button
+5. Click on 'Languages' in the sidebar
+6. Select Hindi
+7. Check Hindi article of India opens with correct title</t>
   </si>
 </sst>
 </file>
@@ -649,7 +991,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="21">
+  <cellXfs count="31">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -682,6 +1024,39 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -705,9 +1080,6 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -985,77 +1357,77 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:H131"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="11.33203125" customWidth="1"/>
-    <col min="2" max="2" width="15.44140625" customWidth="1"/>
-    <col min="3" max="3" width="20.44140625" customWidth="1"/>
-    <col min="4" max="4" width="23.88671875" customWidth="1"/>
-    <col min="5" max="5" width="24.44140625" customWidth="1"/>
-    <col min="6" max="6" width="40.44140625" style="11" customWidth="1"/>
-    <col min="7" max="7" width="20.6640625" customWidth="1"/>
-    <col min="8" max="8" width="31.5546875" customWidth="1"/>
+    <col min="1" max="1" width="11.28515625" customWidth="1"/>
+    <col min="2" max="2" width="15.42578125" customWidth="1"/>
+    <col min="3" max="3" width="20.42578125" customWidth="1"/>
+    <col min="4" max="4" width="23.85546875" customWidth="1"/>
+    <col min="5" max="5" width="24.42578125" customWidth="1"/>
+    <col min="6" max="6" width="40.42578125" style="11" customWidth="1"/>
+    <col min="7" max="7" width="20.7109375" customWidth="1"/>
+    <col min="8" max="8" width="31.5703125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:8">
-      <c r="A1" s="12" t="s">
+      <c r="A1" s="23" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="13"/>
-      <c r="C1" s="13"/>
-      <c r="D1" s="13"/>
-      <c r="E1" s="13"/>
-      <c r="F1" s="13"/>
-      <c r="G1" s="13"/>
-      <c r="H1" s="13"/>
+      <c r="B1" s="24"/>
+      <c r="C1" s="24"/>
+      <c r="D1" s="24"/>
+      <c r="E1" s="24"/>
+      <c r="F1" s="24"/>
+      <c r="G1" s="24"/>
+      <c r="H1" s="24"/>
     </row>
     <row r="2" spans="1:8">
-      <c r="A2" s="12"/>
-      <c r="B2" s="13"/>
-      <c r="C2" s="13"/>
-      <c r="D2" s="13"/>
-      <c r="E2" s="13"/>
-      <c r="F2" s="13"/>
-      <c r="G2" s="13"/>
-      <c r="H2" s="13"/>
+      <c r="A2" s="23"/>
+      <c r="B2" s="24"/>
+      <c r="C2" s="24"/>
+      <c r="D2" s="24"/>
+      <c r="E2" s="24"/>
+      <c r="F2" s="24"/>
+      <c r="G2" s="24"/>
+      <c r="H2" s="24"/>
     </row>
     <row r="3" spans="1:8">
-      <c r="A3" s="13"/>
-      <c r="B3" s="13"/>
-      <c r="C3" s="13"/>
-      <c r="D3" s="13"/>
-      <c r="E3" s="13"/>
-      <c r="F3" s="13"/>
-      <c r="G3" s="13"/>
-      <c r="H3" s="13"/>
+      <c r="A3" s="24"/>
+      <c r="B3" s="24"/>
+      <c r="C3" s="24"/>
+      <c r="D3" s="24"/>
+      <c r="E3" s="24"/>
+      <c r="F3" s="24"/>
+      <c r="G3" s="24"/>
+      <c r="H3" s="24"/>
     </row>
     <row r="4" spans="1:8">
-      <c r="A4" s="14" t="s">
+      <c r="A4" s="25" t="s">
         <v>1</v>
       </c>
-      <c r="B4" s="13"/>
-      <c r="C4" s="15" t="s">
+      <c r="B4" s="24"/>
+      <c r="C4" s="26" t="s">
         <v>2</v>
       </c>
-      <c r="D4" s="13"/>
-      <c r="E4" s="13"/>
-      <c r="F4" s="13" t="s">
+      <c r="D4" s="24"/>
+      <c r="E4" s="24"/>
+      <c r="F4" s="24" t="s">
         <v>3</v>
       </c>
-      <c r="G4" s="13"/>
-      <c r="H4" s="13"/>
+      <c r="G4" s="24"/>
+      <c r="H4" s="24"/>
     </row>
     <row r="5" spans="1:8">
-      <c r="A5" s="13"/>
-      <c r="B5" s="13"/>
-      <c r="C5" s="13"/>
-      <c r="D5" s="13"/>
-      <c r="E5" s="13"/>
-      <c r="F5" s="13"/>
-      <c r="G5" s="13"/>
-      <c r="H5" s="13"/>
-    </row>
-    <row r="6" spans="1:8" ht="40.799999999999997" customHeight="1">
+      <c r="A5" s="24"/>
+      <c r="B5" s="24"/>
+      <c r="C5" s="24"/>
+      <c r="D5" s="24"/>
+      <c r="E5" s="24"/>
+      <c r="F5" s="24"/>
+      <c r="G5" s="24"/>
+      <c r="H5" s="24"/>
+    </row>
+    <row r="6" spans="1:8" ht="40.9" customHeight="1">
       <c r="A6" s="2" t="s">
         <v>4</v>
       </c>
@@ -1081,7 +1453,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="7" spans="1:8" ht="90">
+    <row r="7" spans="1:8" ht="112.5">
       <c r="A7" s="4">
         <v>1</v>
       </c>
@@ -1107,7 +1479,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="8" spans="1:8" ht="108">
+    <row r="8" spans="1:8" ht="112.5">
       <c r="A8" s="4">
         <v>2</v>
       </c>
@@ -1133,7 +1505,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="9" spans="1:8" ht="90">
+    <row r="9" spans="1:8" ht="112.5">
       <c r="A9" s="4">
         <v>3</v>
       </c>
@@ -1185,7 +1557,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="11" spans="1:8" ht="162">
+    <row r="11" spans="1:8" ht="168.75">
       <c r="A11" s="4">
         <v>5</v>
       </c>
@@ -1211,7 +1583,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="12" spans="1:8" ht="162">
+    <row r="12" spans="1:8" ht="168.75">
       <c r="A12" s="4">
         <v>6</v>
       </c>
@@ -1237,7 +1609,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="13" spans="1:8" ht="108">
+    <row r="13" spans="1:8" ht="112.5">
       <c r="A13" s="4">
         <v>7</v>
       </c>
@@ -1263,7 +1635,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="14" spans="1:8" ht="144">
+    <row r="14" spans="1:8" ht="150">
       <c r="A14" s="4">
         <v>8</v>
       </c>
@@ -1289,7 +1661,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="15" spans="1:8" ht="126">
+    <row r="15" spans="1:8" ht="131.25">
       <c r="A15" s="4">
         <v>9</v>
       </c>
@@ -1315,7 +1687,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="16" spans="1:8" ht="126">
+    <row r="16" spans="1:8" ht="150">
       <c r="A16" s="7">
         <v>10</v>
       </c>
@@ -1341,7 +1713,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="17" spans="1:8" ht="234">
+    <row r="17" spans="1:8" ht="243.75">
       <c r="A17" s="7">
         <v>11</v>
       </c>
@@ -1367,7 +1739,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="18" spans="1:8" ht="252">
+    <row r="18" spans="1:8" ht="262.5">
       <c r="A18" s="7">
         <v>12</v>
       </c>
@@ -1393,7 +1765,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="19" spans="1:8" s="7" customFormat="1" ht="198">
+    <row r="19" spans="1:8" s="7" customFormat="1" ht="243.75">
       <c r="A19" s="7">
         <v>13</v>
       </c>
@@ -1419,7 +1791,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="20" spans="1:8" s="7" customFormat="1" ht="306">
+    <row r="20" spans="1:8" s="7" customFormat="1" ht="318.75">
       <c r="A20" s="7">
         <v>14</v>
       </c>
@@ -1445,7 +1817,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="21" spans="1:8" ht="36">
+    <row r="21" spans="1:8" ht="56.25">
       <c r="A21" s="7">
         <v>15</v>
       </c>
@@ -1469,7 +1841,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="22" spans="1:8" ht="18">
+    <row r="22" spans="1:8" ht="18.75">
       <c r="A22" s="7"/>
       <c r="B22" s="7"/>
       <c r="C22" s="7"/>
@@ -1479,7 +1851,7 @@
       <c r="G22" s="7"/>
       <c r="H22" s="4"/>
     </row>
-    <row r="23" spans="1:8" ht="18">
+    <row r="23" spans="1:8" ht="18.75">
       <c r="A23" s="7"/>
       <c r="B23" s="7"/>
       <c r="C23" s="7"/>
@@ -1489,7 +1861,7 @@
       <c r="G23" s="7"/>
       <c r="H23" s="4"/>
     </row>
-    <row r="24" spans="1:8" ht="18">
+    <row r="24" spans="1:8" ht="18.75">
       <c r="A24" s="4"/>
       <c r="B24" s="4"/>
       <c r="C24" s="4"/>
@@ -1499,7 +1871,7 @@
       <c r="G24" s="4"/>
       <c r="H24" s="4"/>
     </row>
-    <row r="25" spans="1:8" ht="18">
+    <row r="25" spans="1:8" ht="18.75">
       <c r="A25" s="4"/>
       <c r="B25" s="4"/>
       <c r="C25" s="4"/>
@@ -1509,7 +1881,7 @@
       <c r="G25" s="4"/>
       <c r="H25" s="4"/>
     </row>
-    <row r="26" spans="1:8" ht="18">
+    <row r="26" spans="1:8" ht="18.75">
       <c r="A26" s="4"/>
       <c r="B26" s="4"/>
       <c r="C26" s="4"/>
@@ -1519,7 +1891,7 @@
       <c r="G26" s="4"/>
       <c r="H26" s="4"/>
     </row>
-    <row r="27" spans="1:8" ht="18">
+    <row r="27" spans="1:8" ht="18.75">
       <c r="A27" s="4"/>
       <c r="B27" s="4"/>
       <c r="C27" s="4"/>
@@ -1529,7 +1901,7 @@
       <c r="G27" s="4"/>
       <c r="H27" s="4"/>
     </row>
-    <row r="28" spans="1:8" ht="18">
+    <row r="28" spans="1:8" ht="18.75">
       <c r="A28" s="4"/>
       <c r="B28" s="4"/>
       <c r="C28" s="4"/>
@@ -1539,7 +1911,7 @@
       <c r="G28" s="4"/>
       <c r="H28" s="4"/>
     </row>
-    <row r="29" spans="1:8" ht="18">
+    <row r="29" spans="1:8" ht="18.75">
       <c r="A29" s="4"/>
       <c r="B29" s="4"/>
       <c r="C29" s="4"/>
@@ -1549,7 +1921,7 @@
       <c r="G29" s="4"/>
       <c r="H29" s="4"/>
     </row>
-    <row r="30" spans="1:8" ht="18">
+    <row r="30" spans="1:8" ht="18.75">
       <c r="A30" s="4"/>
       <c r="B30" s="4"/>
       <c r="C30" s="4"/>
@@ -1559,7 +1931,7 @@
       <c r="G30" s="4"/>
       <c r="H30" s="4"/>
     </row>
-    <row r="31" spans="1:8" ht="18">
+    <row r="31" spans="1:8" ht="18.75">
       <c r="A31" s="4"/>
       <c r="B31" s="4"/>
       <c r="C31" s="4"/>
@@ -1569,7 +1941,7 @@
       <c r="G31" s="4"/>
       <c r="H31" s="4"/>
     </row>
-    <row r="32" spans="1:8" ht="18">
+    <row r="32" spans="1:8" ht="18.75">
       <c r="A32" s="4"/>
       <c r="B32" s="4"/>
       <c r="C32" s="4"/>
@@ -1579,7 +1951,7 @@
       <c r="G32" s="4"/>
       <c r="H32" s="4"/>
     </row>
-    <row r="33" spans="1:8" ht="18">
+    <row r="33" spans="1:8" ht="18.75">
       <c r="A33" s="4"/>
       <c r="B33" s="4"/>
       <c r="C33" s="4"/>
@@ -1589,7 +1961,7 @@
       <c r="G33" s="4"/>
       <c r="H33" s="4"/>
     </row>
-    <row r="34" spans="1:8" ht="18">
+    <row r="34" spans="1:8" ht="18.75">
       <c r="A34" s="4"/>
       <c r="B34" s="4"/>
       <c r="C34" s="4"/>
@@ -1599,7 +1971,7 @@
       <c r="G34" s="4"/>
       <c r="H34" s="4"/>
     </row>
-    <row r="35" spans="1:8" ht="18">
+    <row r="35" spans="1:8" ht="18.75">
       <c r="A35" s="4"/>
       <c r="B35" s="4"/>
       <c r="C35" s="4"/>
@@ -1609,7 +1981,7 @@
       <c r="G35" s="4"/>
       <c r="H35" s="4"/>
     </row>
-    <row r="36" spans="1:8" ht="18">
+    <row r="36" spans="1:8" ht="18.75">
       <c r="A36" s="4"/>
       <c r="B36" s="4"/>
       <c r="C36" s="4"/>
@@ -1619,7 +1991,7 @@
       <c r="G36" s="4"/>
       <c r="H36" s="4"/>
     </row>
-    <row r="37" spans="1:8" ht="18">
+    <row r="37" spans="1:8" ht="18.75">
       <c r="A37" s="4"/>
       <c r="B37" s="4"/>
       <c r="C37" s="4"/>
@@ -1629,7 +2001,7 @@
       <c r="G37" s="4"/>
       <c r="H37" s="4"/>
     </row>
-    <row r="38" spans="1:8" ht="18">
+    <row r="38" spans="1:8" ht="18.75">
       <c r="A38" s="4"/>
       <c r="B38" s="4"/>
       <c r="C38" s="4"/>
@@ -1639,7 +2011,7 @@
       <c r="G38" s="4"/>
       <c r="H38" s="4"/>
     </row>
-    <row r="39" spans="1:8" ht="18">
+    <row r="39" spans="1:8" ht="18.75">
       <c r="A39" s="4"/>
       <c r="B39" s="4"/>
       <c r="C39" s="4"/>
@@ -1649,7 +2021,7 @@
       <c r="G39" s="4"/>
       <c r="H39" s="4"/>
     </row>
-    <row r="40" spans="1:8" ht="15.6">
+    <row r="40" spans="1:8" ht="15.75">
       <c r="A40" s="6"/>
       <c r="B40" s="6"/>
       <c r="C40" s="6"/>
@@ -1659,7 +2031,7 @@
       <c r="G40" s="6"/>
       <c r="H40" s="6"/>
     </row>
-    <row r="41" spans="1:8" ht="15.6">
+    <row r="41" spans="1:8" ht="15.75">
       <c r="A41" s="6"/>
       <c r="B41" s="6"/>
       <c r="C41" s="6"/>
@@ -1669,7 +2041,7 @@
       <c r="G41" s="6"/>
       <c r="H41" s="6"/>
     </row>
-    <row r="42" spans="1:8" ht="15.6">
+    <row r="42" spans="1:8" ht="15.75">
       <c r="A42" s="6"/>
       <c r="B42" s="6"/>
       <c r="C42" s="6"/>
@@ -1679,7 +2051,7 @@
       <c r="G42" s="6"/>
       <c r="H42" s="6"/>
     </row>
-    <row r="43" spans="1:8" ht="15.6">
+    <row r="43" spans="1:8" ht="15.75">
       <c r="A43" s="6"/>
       <c r="B43" s="6"/>
       <c r="C43" s="6"/>
@@ -1689,7 +2061,7 @@
       <c r="G43" s="6"/>
       <c r="H43" s="6"/>
     </row>
-    <row r="44" spans="1:8" ht="15.6">
+    <row r="44" spans="1:8" ht="15.75">
       <c r="A44" s="6"/>
       <c r="B44" s="6"/>
       <c r="C44" s="6"/>
@@ -1699,7 +2071,7 @@
       <c r="G44" s="6"/>
       <c r="H44" s="6"/>
     </row>
-    <row r="45" spans="1:8" ht="15.6">
+    <row r="45" spans="1:8" ht="15.75">
       <c r="A45" s="6"/>
       <c r="B45" s="6"/>
       <c r="C45" s="6"/>
@@ -1709,7 +2081,7 @@
       <c r="G45" s="6"/>
       <c r="H45" s="6"/>
     </row>
-    <row r="46" spans="1:8" ht="15.6">
+    <row r="46" spans="1:8" ht="15.75">
       <c r="A46" s="6"/>
       <c r="B46" s="6"/>
       <c r="C46" s="6"/>
@@ -1719,7 +2091,7 @@
       <c r="G46" s="6"/>
       <c r="H46" s="6"/>
     </row>
-    <row r="47" spans="1:8" ht="15.6">
+    <row r="47" spans="1:8" ht="15.75">
       <c r="A47" s="6"/>
       <c r="B47" s="6"/>
       <c r="C47" s="6"/>
@@ -1729,7 +2101,7 @@
       <c r="G47" s="6"/>
       <c r="H47" s="6"/>
     </row>
-    <row r="48" spans="1:8" ht="15.6">
+    <row r="48" spans="1:8" ht="15.75">
       <c r="A48" s="6"/>
       <c r="B48" s="6"/>
       <c r="C48" s="6"/>
@@ -1739,7 +2111,7 @@
       <c r="G48" s="6"/>
       <c r="H48" s="6"/>
     </row>
-    <row r="49" spans="1:8" ht="15.6">
+    <row r="49" spans="1:8" ht="15.75">
       <c r="A49" s="6"/>
       <c r="B49" s="6"/>
       <c r="C49" s="6"/>
@@ -1749,7 +2121,7 @@
       <c r="G49" s="6"/>
       <c r="H49" s="6"/>
     </row>
-    <row r="50" spans="1:8" ht="15.6">
+    <row r="50" spans="1:8" ht="15.75">
       <c r="A50" s="6"/>
       <c r="B50" s="6"/>
       <c r="C50" s="6"/>
@@ -1759,7 +2131,7 @@
       <c r="G50" s="6"/>
       <c r="H50" s="6"/>
     </row>
-    <row r="51" spans="1:8" ht="15.6">
+    <row r="51" spans="1:8" ht="15.75">
       <c r="A51" s="6"/>
       <c r="B51" s="6"/>
       <c r="C51" s="6"/>
@@ -1769,7 +2141,7 @@
       <c r="G51" s="6"/>
       <c r="H51" s="6"/>
     </row>
-    <row r="52" spans="1:8" ht="15.6">
+    <row r="52" spans="1:8" ht="15.75">
       <c r="A52" s="6"/>
       <c r="B52" s="6"/>
       <c r="C52" s="6"/>
@@ -1779,7 +2151,7 @@
       <c r="G52" s="6"/>
       <c r="H52" s="6"/>
     </row>
-    <row r="53" spans="1:8" ht="15.6">
+    <row r="53" spans="1:8" ht="15.75">
       <c r="A53" s="6"/>
       <c r="B53" s="6"/>
       <c r="C53" s="6"/>
@@ -1789,7 +2161,7 @@
       <c r="G53" s="6"/>
       <c r="H53" s="6"/>
     </row>
-    <row r="54" spans="1:8" ht="15.6">
+    <row r="54" spans="1:8" ht="15.75">
       <c r="A54" s="6"/>
       <c r="B54" s="6"/>
       <c r="C54" s="6"/>
@@ -1799,7 +2171,7 @@
       <c r="G54" s="6"/>
       <c r="H54" s="6"/>
     </row>
-    <row r="55" spans="1:8" ht="15.6">
+    <row r="55" spans="1:8" ht="15.75">
       <c r="A55" s="6"/>
       <c r="B55" s="6"/>
       <c r="C55" s="6"/>
@@ -1809,7 +2181,7 @@
       <c r="G55" s="6"/>
       <c r="H55" s="6"/>
     </row>
-    <row r="56" spans="1:8" ht="15.6">
+    <row r="56" spans="1:8" ht="15.75">
       <c r="A56" s="6"/>
       <c r="B56" s="6"/>
       <c r="C56" s="6"/>
@@ -1819,7 +2191,7 @@
       <c r="G56" s="6"/>
       <c r="H56" s="6"/>
     </row>
-    <row r="57" spans="1:8" ht="15.6">
+    <row r="57" spans="1:8" ht="15.75">
       <c r="A57" s="6"/>
       <c r="B57" s="6"/>
       <c r="C57" s="6"/>
@@ -1829,7 +2201,7 @@
       <c r="G57" s="6"/>
       <c r="H57" s="6"/>
     </row>
-    <row r="58" spans="1:8" ht="15.6">
+    <row r="58" spans="1:8" ht="15.75">
       <c r="A58" s="6"/>
       <c r="B58" s="6"/>
       <c r="C58" s="6"/>
@@ -1839,7 +2211,7 @@
       <c r="G58" s="6"/>
       <c r="H58" s="6"/>
     </row>
-    <row r="59" spans="1:8" ht="15.6">
+    <row r="59" spans="1:8" ht="15.75">
       <c r="A59" s="6"/>
       <c r="B59" s="6"/>
       <c r="C59" s="6"/>
@@ -1849,7 +2221,7 @@
       <c r="G59" s="6"/>
       <c r="H59" s="6"/>
     </row>
-    <row r="60" spans="1:8" ht="15.6">
+    <row r="60" spans="1:8" ht="15.75">
       <c r="A60" s="6"/>
       <c r="B60" s="6"/>
       <c r="C60" s="6"/>
@@ -1859,7 +2231,7 @@
       <c r="G60" s="6"/>
       <c r="H60" s="6"/>
     </row>
-    <row r="61" spans="1:8" ht="15.6">
+    <row r="61" spans="1:8" ht="15.75">
       <c r="A61" s="6"/>
       <c r="B61" s="6"/>
       <c r="C61" s="6"/>
@@ -1869,7 +2241,7 @@
       <c r="G61" s="6"/>
       <c r="H61" s="6"/>
     </row>
-    <row r="62" spans="1:8" ht="15.6">
+    <row r="62" spans="1:8" ht="15.75">
       <c r="A62" s="6"/>
       <c r="B62" s="6"/>
       <c r="C62" s="6"/>
@@ -1879,7 +2251,7 @@
       <c r="G62" s="6"/>
       <c r="H62" s="6"/>
     </row>
-    <row r="63" spans="1:8" ht="15.6">
+    <row r="63" spans="1:8" ht="15.75">
       <c r="A63" s="6"/>
       <c r="B63" s="6"/>
       <c r="C63" s="6"/>
@@ -1889,7 +2261,7 @@
       <c r="G63" s="6"/>
       <c r="H63" s="6"/>
     </row>
-    <row r="64" spans="1:8" ht="15.6">
+    <row r="64" spans="1:8" ht="15.75">
       <c r="A64" s="6"/>
       <c r="B64" s="6"/>
       <c r="C64" s="6"/>
@@ -1899,7 +2271,7 @@
       <c r="G64" s="6"/>
       <c r="H64" s="6"/>
     </row>
-    <row r="65" spans="1:8" ht="15.6">
+    <row r="65" spans="1:8" ht="15.75">
       <c r="A65" s="6"/>
       <c r="B65" s="6"/>
       <c r="C65" s="6"/>
@@ -1909,7 +2281,7 @@
       <c r="G65" s="6"/>
       <c r="H65" s="6"/>
     </row>
-    <row r="66" spans="1:8" ht="15.6">
+    <row r="66" spans="1:8" ht="15.75">
       <c r="A66" s="6"/>
       <c r="B66" s="6"/>
       <c r="C66" s="6"/>
@@ -1919,7 +2291,7 @@
       <c r="G66" s="6"/>
       <c r="H66" s="6"/>
     </row>
-    <row r="67" spans="1:8" ht="15.6">
+    <row r="67" spans="1:8" ht="15.75">
       <c r="A67" s="6"/>
       <c r="B67" s="6"/>
       <c r="C67" s="6"/>
@@ -1929,7 +2301,7 @@
       <c r="G67" s="6"/>
       <c r="H67" s="6"/>
     </row>
-    <row r="68" spans="1:8" ht="15.6">
+    <row r="68" spans="1:8" ht="15.75">
       <c r="A68" s="6"/>
       <c r="B68" s="6"/>
       <c r="C68" s="6"/>
@@ -1939,7 +2311,7 @@
       <c r="G68" s="6"/>
       <c r="H68" s="6"/>
     </row>
-    <row r="69" spans="1:8" ht="15.6">
+    <row r="69" spans="1:8" ht="15.75">
       <c r="A69" s="6"/>
       <c r="B69" s="6"/>
       <c r="C69" s="6"/>
@@ -1949,7 +2321,7 @@
       <c r="G69" s="6"/>
       <c r="H69" s="6"/>
     </row>
-    <row r="70" spans="1:8" ht="15.6">
+    <row r="70" spans="1:8" ht="15.75">
       <c r="A70" s="6"/>
       <c r="B70" s="6"/>
       <c r="C70" s="6"/>
@@ -1959,7 +2331,7 @@
       <c r="G70" s="6"/>
       <c r="H70" s="6"/>
     </row>
-    <row r="71" spans="1:8" ht="15.6">
+    <row r="71" spans="1:8" ht="15.75">
       <c r="A71" s="6"/>
       <c r="B71" s="6"/>
       <c r="C71" s="6"/>
@@ -1969,7 +2341,7 @@
       <c r="G71" s="6"/>
       <c r="H71" s="6"/>
     </row>
-    <row r="72" spans="1:8" ht="15.6">
+    <row r="72" spans="1:8" ht="15.75">
       <c r="A72" s="6"/>
       <c r="B72" s="6"/>
       <c r="C72" s="6"/>
@@ -1979,7 +2351,7 @@
       <c r="G72" s="6"/>
       <c r="H72" s="6"/>
     </row>
-    <row r="73" spans="1:8" ht="15.6">
+    <row r="73" spans="1:8" ht="15.75">
       <c r="A73" s="6"/>
       <c r="B73" s="6"/>
       <c r="C73" s="6"/>
@@ -1989,7 +2361,7 @@
       <c r="G73" s="6"/>
       <c r="H73" s="6"/>
     </row>
-    <row r="74" spans="1:8" ht="15.6">
+    <row r="74" spans="1:8" ht="15.75">
       <c r="A74" s="6"/>
       <c r="B74" s="6"/>
       <c r="C74" s="6"/>
@@ -1999,7 +2371,7 @@
       <c r="G74" s="6"/>
       <c r="H74" s="6"/>
     </row>
-    <row r="75" spans="1:8" ht="15.6">
+    <row r="75" spans="1:8" ht="15.75">
       <c r="A75" s="6"/>
       <c r="B75" s="6"/>
       <c r="C75" s="6"/>
@@ -2009,7 +2381,7 @@
       <c r="G75" s="6"/>
       <c r="H75" s="6"/>
     </row>
-    <row r="76" spans="1:8" ht="15.6">
+    <row r="76" spans="1:8" ht="15.75">
       <c r="A76" s="6"/>
       <c r="B76" s="6"/>
       <c r="C76" s="6"/>
@@ -2019,7 +2391,7 @@
       <c r="G76" s="6"/>
       <c r="H76" s="6"/>
     </row>
-    <row r="77" spans="1:8" ht="15.6">
+    <row r="77" spans="1:8" ht="15.75">
       <c r="A77" s="6"/>
       <c r="B77" s="6"/>
       <c r="C77" s="6"/>
@@ -2029,7 +2401,7 @@
       <c r="G77" s="6"/>
       <c r="H77" s="6"/>
     </row>
-    <row r="78" spans="1:8" ht="15.6">
+    <row r="78" spans="1:8" ht="15.75">
       <c r="A78" s="6"/>
       <c r="B78" s="6"/>
       <c r="C78" s="6"/>
@@ -2039,7 +2411,7 @@
       <c r="G78" s="6"/>
       <c r="H78" s="6"/>
     </row>
-    <row r="79" spans="1:8" ht="15.6">
+    <row r="79" spans="1:8" ht="15.75">
       <c r="A79" s="6"/>
       <c r="B79" s="6"/>
       <c r="C79" s="6"/>
@@ -2049,7 +2421,7 @@
       <c r="G79" s="6"/>
       <c r="H79" s="6"/>
     </row>
-    <row r="80" spans="1:8" ht="15.6">
+    <row r="80" spans="1:8" ht="15.75">
       <c r="A80" s="6"/>
       <c r="B80" s="6"/>
       <c r="C80" s="6"/>
@@ -2059,7 +2431,7 @@
       <c r="G80" s="6"/>
       <c r="H80" s="6"/>
     </row>
-    <row r="81" spans="1:8" ht="15.6">
+    <row r="81" spans="1:8" ht="15.75">
       <c r="A81" s="6"/>
       <c r="B81" s="6"/>
       <c r="C81" s="6"/>
@@ -2069,7 +2441,7 @@
       <c r="G81" s="6"/>
       <c r="H81" s="6"/>
     </row>
-    <row r="82" spans="1:8" ht="15.6">
+    <row r="82" spans="1:8" ht="15.75">
       <c r="A82" s="6"/>
       <c r="B82" s="6"/>
       <c r="C82" s="6"/>
@@ -2079,7 +2451,7 @@
       <c r="G82" s="6"/>
       <c r="H82" s="6"/>
     </row>
-    <row r="83" spans="1:8" ht="15.6">
+    <row r="83" spans="1:8" ht="15.75">
       <c r="A83" s="6"/>
       <c r="B83" s="6"/>
       <c r="C83" s="6"/>
@@ -2089,7 +2461,7 @@
       <c r="G83" s="6"/>
       <c r="H83" s="6"/>
     </row>
-    <row r="84" spans="1:8" ht="15.6">
+    <row r="84" spans="1:8" ht="15.75">
       <c r="A84" s="6"/>
       <c r="B84" s="6"/>
       <c r="C84" s="6"/>
@@ -2099,7 +2471,7 @@
       <c r="G84" s="6"/>
       <c r="H84" s="6"/>
     </row>
-    <row r="85" spans="1:8" ht="15.6">
+    <row r="85" spans="1:8" ht="15.75">
       <c r="A85" s="6"/>
       <c r="B85" s="6"/>
       <c r="C85" s="6"/>
@@ -2109,7 +2481,7 @@
       <c r="G85" s="6"/>
       <c r="H85" s="6"/>
     </row>
-    <row r="86" spans="1:8" ht="15.6">
+    <row r="86" spans="1:8" ht="15.75">
       <c r="A86" s="6"/>
       <c r="B86" s="6"/>
       <c r="C86" s="6"/>
@@ -2119,7 +2491,7 @@
       <c r="G86" s="6"/>
       <c r="H86" s="6"/>
     </row>
-    <row r="87" spans="1:8" ht="15.6">
+    <row r="87" spans="1:8" ht="15.75">
       <c r="A87" s="6"/>
       <c r="B87" s="6"/>
       <c r="C87" s="6"/>
@@ -2129,7 +2501,7 @@
       <c r="G87" s="6"/>
       <c r="H87" s="6"/>
     </row>
-    <row r="88" spans="1:8" ht="15.6">
+    <row r="88" spans="1:8" ht="15.75">
       <c r="A88" s="6"/>
       <c r="B88" s="6"/>
       <c r="C88" s="6"/>
@@ -2139,7 +2511,7 @@
       <c r="G88" s="6"/>
       <c r="H88" s="6"/>
     </row>
-    <row r="89" spans="1:8" ht="15.6">
+    <row r="89" spans="1:8" ht="15.75">
       <c r="A89" s="6"/>
       <c r="B89" s="6"/>
       <c r="C89" s="6"/>
@@ -2149,7 +2521,7 @@
       <c r="G89" s="6"/>
       <c r="H89" s="6"/>
     </row>
-    <row r="90" spans="1:8" ht="15.6">
+    <row r="90" spans="1:8" ht="15.75">
       <c r="A90" s="6"/>
       <c r="B90" s="6"/>
       <c r="C90" s="6"/>
@@ -2159,7 +2531,7 @@
       <c r="G90" s="6"/>
       <c r="H90" s="6"/>
     </row>
-    <row r="91" spans="1:8" ht="15.6">
+    <row r="91" spans="1:8" ht="15.75">
       <c r="A91" s="6"/>
       <c r="B91" s="6"/>
       <c r="C91" s="6"/>
@@ -2169,7 +2541,7 @@
       <c r="G91" s="6"/>
       <c r="H91" s="6"/>
     </row>
-    <row r="92" spans="1:8" ht="15.6">
+    <row r="92" spans="1:8" ht="15.75">
       <c r="A92" s="6"/>
       <c r="B92" s="6"/>
       <c r="C92" s="6"/>
@@ -2179,7 +2551,7 @@
       <c r="G92" s="6"/>
       <c r="H92" s="6"/>
     </row>
-    <row r="93" spans="1:8" ht="15.6">
+    <row r="93" spans="1:8" ht="15.75">
       <c r="A93" s="6"/>
       <c r="B93" s="6"/>
       <c r="C93" s="6"/>
@@ -2189,7 +2561,7 @@
       <c r="G93" s="6"/>
       <c r="H93" s="6"/>
     </row>
-    <row r="94" spans="1:8" ht="15.6">
+    <row r="94" spans="1:8" ht="15.75">
       <c r="A94" s="6"/>
       <c r="B94" s="6"/>
       <c r="C94" s="6"/>
@@ -2199,7 +2571,7 @@
       <c r="G94" s="6"/>
       <c r="H94" s="6"/>
     </row>
-    <row r="95" spans="1:8" ht="15.6">
+    <row r="95" spans="1:8" ht="15.75">
       <c r="A95" s="6"/>
       <c r="B95" s="6"/>
       <c r="C95" s="6"/>
@@ -2209,7 +2581,7 @@
       <c r="G95" s="6"/>
       <c r="H95" s="6"/>
     </row>
-    <row r="96" spans="1:8" ht="15.6">
+    <row r="96" spans="1:8" ht="15.75">
       <c r="A96" s="6"/>
       <c r="B96" s="6"/>
       <c r="C96" s="6"/>
@@ -2219,7 +2591,7 @@
       <c r="G96" s="6"/>
       <c r="H96" s="6"/>
     </row>
-    <row r="97" spans="1:8" ht="15.6">
+    <row r="97" spans="1:8" ht="15.75">
       <c r="A97" s="6"/>
       <c r="B97" s="6"/>
       <c r="C97" s="6"/>
@@ -2229,7 +2601,7 @@
       <c r="G97" s="6"/>
       <c r="H97" s="6"/>
     </row>
-    <row r="98" spans="1:8" ht="15.6">
+    <row r="98" spans="1:8" ht="15.75">
       <c r="A98" s="6"/>
       <c r="B98" s="6"/>
       <c r="C98" s="6"/>
@@ -2239,7 +2611,7 @@
       <c r="G98" s="6"/>
       <c r="H98" s="6"/>
     </row>
-    <row r="99" spans="1:8" ht="15.6">
+    <row r="99" spans="1:8" ht="15.75">
       <c r="A99" s="6"/>
       <c r="B99" s="6"/>
       <c r="C99" s="6"/>
@@ -2249,7 +2621,7 @@
       <c r="G99" s="6"/>
       <c r="H99" s="6"/>
     </row>
-    <row r="100" spans="1:8" ht="15.6">
+    <row r="100" spans="1:8" ht="15.75">
       <c r="A100" s="6"/>
       <c r="B100" s="6"/>
       <c r="C100" s="6"/>
@@ -2259,7 +2631,7 @@
       <c r="G100" s="6"/>
       <c r="H100" s="6"/>
     </row>
-    <row r="101" spans="1:8" ht="15.6">
+    <row r="101" spans="1:8" ht="15.75">
       <c r="A101" s="6"/>
       <c r="B101" s="6"/>
       <c r="C101" s="6"/>
@@ -2269,7 +2641,7 @@
       <c r="G101" s="6"/>
       <c r="H101" s="6"/>
     </row>
-    <row r="102" spans="1:8" ht="15.6">
+    <row r="102" spans="1:8" ht="15.75">
       <c r="A102" s="6"/>
       <c r="B102" s="6"/>
       <c r="C102" s="6"/>
@@ -2279,7 +2651,7 @@
       <c r="G102" s="6"/>
       <c r="H102" s="6"/>
     </row>
-    <row r="103" spans="1:8" ht="15.6">
+    <row r="103" spans="1:8" ht="15.75">
       <c r="A103" s="6"/>
       <c r="B103" s="6"/>
       <c r="C103" s="6"/>
@@ -2289,7 +2661,7 @@
       <c r="G103" s="6"/>
       <c r="H103" s="6"/>
     </row>
-    <row r="104" spans="1:8" ht="15.6">
+    <row r="104" spans="1:8" ht="15.75">
       <c r="A104" s="6"/>
       <c r="B104" s="6"/>
       <c r="C104" s="6"/>
@@ -2299,7 +2671,7 @@
       <c r="G104" s="6"/>
       <c r="H104" s="6"/>
     </row>
-    <row r="105" spans="1:8" ht="15.6">
+    <row r="105" spans="1:8" ht="15.75">
       <c r="A105" s="6"/>
       <c r="B105" s="6"/>
       <c r="C105" s="6"/>
@@ -2309,7 +2681,7 @@
       <c r="G105" s="6"/>
       <c r="H105" s="6"/>
     </row>
-    <row r="106" spans="1:8" ht="15.6">
+    <row r="106" spans="1:8" ht="15.75">
       <c r="A106" s="6"/>
       <c r="B106" s="6"/>
       <c r="C106" s="6"/>
@@ -2319,7 +2691,7 @@
       <c r="G106" s="6"/>
       <c r="H106" s="6"/>
     </row>
-    <row r="107" spans="1:8" ht="15.6">
+    <row r="107" spans="1:8" ht="15.75">
       <c r="A107" s="6"/>
       <c r="B107" s="6"/>
       <c r="C107" s="6"/>
@@ -2329,7 +2701,7 @@
       <c r="G107" s="6"/>
       <c r="H107" s="6"/>
     </row>
-    <row r="108" spans="1:8" ht="15.6">
+    <row r="108" spans="1:8" ht="15.75">
       <c r="A108" s="6"/>
       <c r="B108" s="6"/>
       <c r="C108" s="6"/>
@@ -2339,7 +2711,7 @@
       <c r="G108" s="6"/>
       <c r="H108" s="6"/>
     </row>
-    <row r="109" spans="1:8" ht="15.6">
+    <row r="109" spans="1:8" ht="15.75">
       <c r="A109" s="6"/>
       <c r="B109" s="6"/>
       <c r="C109" s="6"/>
@@ -2349,7 +2721,7 @@
       <c r="G109" s="6"/>
       <c r="H109" s="6"/>
     </row>
-    <row r="110" spans="1:8" ht="15.6">
+    <row r="110" spans="1:8" ht="15.75">
       <c r="A110" s="6"/>
       <c r="B110" s="6"/>
       <c r="C110" s="6"/>
@@ -2359,7 +2731,7 @@
       <c r="G110" s="6"/>
       <c r="H110" s="6"/>
     </row>
-    <row r="111" spans="1:8" ht="15.6">
+    <row r="111" spans="1:8" ht="15.75">
       <c r="A111" s="6"/>
       <c r="B111" s="6"/>
       <c r="C111" s="6"/>
@@ -2369,7 +2741,7 @@
       <c r="G111" s="6"/>
       <c r="H111" s="6"/>
     </row>
-    <row r="112" spans="1:8" ht="15.6">
+    <row r="112" spans="1:8" ht="15.75">
       <c r="A112" s="6"/>
       <c r="B112" s="6"/>
       <c r="C112" s="6"/>
@@ -2379,7 +2751,7 @@
       <c r="G112" s="6"/>
       <c r="H112" s="6"/>
     </row>
-    <row r="113" spans="1:8" ht="15.6">
+    <row r="113" spans="1:8" ht="15.75">
       <c r="A113" s="6"/>
       <c r="B113" s="6"/>
       <c r="C113" s="6"/>
@@ -2389,7 +2761,7 @@
       <c r="G113" s="6"/>
       <c r="H113" s="6"/>
     </row>
-    <row r="114" spans="1:8" ht="15.6">
+    <row r="114" spans="1:8" ht="15.75">
       <c r="A114" s="6"/>
       <c r="B114" s="6"/>
       <c r="C114" s="6"/>
@@ -2399,7 +2771,7 @@
       <c r="G114" s="6"/>
       <c r="H114" s="6"/>
     </row>
-    <row r="115" spans="1:8" ht="15.6">
+    <row r="115" spans="1:8" ht="15.75">
       <c r="A115" s="6"/>
       <c r="B115" s="6"/>
       <c r="C115" s="6"/>
@@ -2409,7 +2781,7 @@
       <c r="G115" s="6"/>
       <c r="H115" s="6"/>
     </row>
-    <row r="116" spans="1:8" ht="15.6">
+    <row r="116" spans="1:8" ht="15.75">
       <c r="A116" s="6"/>
       <c r="B116" s="6"/>
       <c r="C116" s="6"/>
@@ -2419,7 +2791,7 @@
       <c r="G116" s="6"/>
       <c r="H116" s="6"/>
     </row>
-    <row r="117" spans="1:8" ht="15.6">
+    <row r="117" spans="1:8" ht="15.75">
       <c r="A117" s="6"/>
       <c r="B117" s="6"/>
       <c r="C117" s="6"/>
@@ -2429,7 +2801,7 @@
       <c r="G117" s="6"/>
       <c r="H117" s="6"/>
     </row>
-    <row r="118" spans="1:8" ht="15.6">
+    <row r="118" spans="1:8" ht="15.75">
       <c r="A118" s="6"/>
       <c r="B118" s="6"/>
       <c r="C118" s="6"/>
@@ -2439,7 +2811,7 @@
       <c r="G118" s="6"/>
       <c r="H118" s="6"/>
     </row>
-    <row r="119" spans="1:8" ht="15.6">
+    <row r="119" spans="1:8" ht="15.75">
       <c r="A119" s="6"/>
       <c r="B119" s="6"/>
       <c r="C119" s="6"/>
@@ -2449,7 +2821,7 @@
       <c r="G119" s="6"/>
       <c r="H119" s="6"/>
     </row>
-    <row r="120" spans="1:8" ht="15.6">
+    <row r="120" spans="1:8" ht="15.75">
       <c r="A120" s="6"/>
       <c r="B120" s="6"/>
       <c r="C120" s="6"/>
@@ -2459,7 +2831,7 @@
       <c r="G120" s="6"/>
       <c r="H120" s="6"/>
     </row>
-    <row r="121" spans="1:8" ht="15.6">
+    <row r="121" spans="1:8" ht="15.75">
       <c r="A121" s="6"/>
       <c r="B121" s="6"/>
       <c r="C121" s="6"/>
@@ -2469,7 +2841,7 @@
       <c r="G121" s="6"/>
       <c r="H121" s="6"/>
     </row>
-    <row r="122" spans="1:8" ht="15.6">
+    <row r="122" spans="1:8" ht="15.75">
       <c r="A122" s="6"/>
       <c r="B122" s="6"/>
       <c r="C122" s="6"/>
@@ -2479,7 +2851,7 @@
       <c r="G122" s="6"/>
       <c r="H122" s="6"/>
     </row>
-    <row r="123" spans="1:8" ht="15.6">
+    <row r="123" spans="1:8" ht="15.75">
       <c r="A123" s="6"/>
       <c r="B123" s="6"/>
       <c r="C123" s="6"/>
@@ -2489,7 +2861,7 @@
       <c r="G123" s="6"/>
       <c r="H123" s="6"/>
     </row>
-    <row r="124" spans="1:8" ht="15.6">
+    <row r="124" spans="1:8" ht="15.75">
       <c r="A124" s="6"/>
       <c r="B124" s="6"/>
       <c r="C124" s="6"/>
@@ -2499,7 +2871,7 @@
       <c r="G124" s="6"/>
       <c r="H124" s="6"/>
     </row>
-    <row r="125" spans="1:8" ht="15.6">
+    <row r="125" spans="1:8" ht="15.75">
       <c r="A125" s="6"/>
       <c r="B125" s="6"/>
       <c r="C125" s="6"/>
@@ -2509,7 +2881,7 @@
       <c r="G125" s="6"/>
       <c r="H125" s="6"/>
     </row>
-    <row r="126" spans="1:8" ht="15.6">
+    <row r="126" spans="1:8" ht="15.75">
       <c r="A126" s="6"/>
       <c r="B126" s="6"/>
       <c r="C126" s="6"/>
@@ -2519,7 +2891,7 @@
       <c r="G126" s="6"/>
       <c r="H126" s="6"/>
     </row>
-    <row r="127" spans="1:8" ht="15.6">
+    <row r="127" spans="1:8" ht="15.75">
       <c r="A127" s="6"/>
       <c r="B127" s="6"/>
       <c r="C127" s="6"/>
@@ -2529,7 +2901,7 @@
       <c r="G127" s="6"/>
       <c r="H127" s="6"/>
     </row>
-    <row r="128" spans="1:8" ht="15.6">
+    <row r="128" spans="1:8" ht="15.75">
       <c r="A128" s="6"/>
       <c r="B128" s="6"/>
       <c r="C128" s="6"/>
@@ -2539,7 +2911,7 @@
       <c r="G128" s="6"/>
       <c r="H128" s="6"/>
     </row>
-    <row r="129" spans="1:8" ht="15.6">
+    <row r="129" spans="1:8" ht="15.75">
       <c r="A129" s="6"/>
       <c r="B129" s="6"/>
       <c r="C129" s="6"/>
@@ -2549,7 +2921,7 @@
       <c r="G129" s="6"/>
       <c r="H129" s="6"/>
     </row>
-    <row r="130" spans="1:8" ht="15.6">
+    <row r="130" spans="1:8" ht="15.75">
       <c r="A130" s="6"/>
       <c r="B130" s="6"/>
       <c r="C130" s="6"/>
@@ -2559,7 +2931,7 @@
       <c r="G130" s="6"/>
       <c r="H130" s="6"/>
     </row>
-    <row r="131" spans="1:8" ht="15.6">
+    <row r="131" spans="1:8" ht="15.75">
       <c r="A131" s="6"/>
       <c r="B131" s="6"/>
       <c r="C131" s="6"/>
@@ -2584,77 +2956,77 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:H16"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="14.6640625" customWidth="1"/>
-    <col min="2" max="2" width="20.44140625" customWidth="1"/>
-    <col min="3" max="3" width="32.33203125" customWidth="1"/>
-    <col min="4" max="4" width="23.44140625" customWidth="1"/>
-    <col min="5" max="5" width="22.88671875" customWidth="1"/>
-    <col min="6" max="6" width="21.109375" customWidth="1"/>
-    <col min="7" max="7" width="22.44140625" customWidth="1"/>
+    <col min="1" max="1" width="14.7109375" customWidth="1"/>
+    <col min="2" max="2" width="20.42578125" customWidth="1"/>
+    <col min="3" max="3" width="32.28515625" customWidth="1"/>
+    <col min="4" max="4" width="23.42578125" customWidth="1"/>
+    <col min="5" max="5" width="22.85546875" customWidth="1"/>
+    <col min="6" max="6" width="21.140625" customWidth="1"/>
+    <col min="7" max="7" width="22.42578125" customWidth="1"/>
     <col min="8" max="8" width="29" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:8">
-      <c r="A1" s="16" t="s">
+      <c r="A1" s="27" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="17"/>
-      <c r="C1" s="17"/>
-      <c r="D1" s="17"/>
-      <c r="E1" s="17"/>
-      <c r="F1" s="17"/>
-      <c r="G1" s="17"/>
-      <c r="H1" s="17"/>
+      <c r="B1" s="28"/>
+      <c r="C1" s="28"/>
+      <c r="D1" s="28"/>
+      <c r="E1" s="28"/>
+      <c r="F1" s="28"/>
+      <c r="G1" s="28"/>
+      <c r="H1" s="28"/>
     </row>
     <row r="2" spans="1:8">
-      <c r="A2" s="16"/>
-      <c r="B2" s="17"/>
-      <c r="C2" s="17"/>
-      <c r="D2" s="17"/>
-      <c r="E2" s="17"/>
-      <c r="F2" s="17"/>
-      <c r="G2" s="17"/>
-      <c r="H2" s="17"/>
+      <c r="A2" s="27"/>
+      <c r="B2" s="28"/>
+      <c r="C2" s="28"/>
+      <c r="D2" s="28"/>
+      <c r="E2" s="28"/>
+      <c r="F2" s="28"/>
+      <c r="G2" s="28"/>
+      <c r="H2" s="28"/>
     </row>
     <row r="3" spans="1:8">
-      <c r="A3" s="17"/>
-      <c r="B3" s="17"/>
-      <c r="C3" s="17"/>
-      <c r="D3" s="17"/>
-      <c r="E3" s="17"/>
-      <c r="F3" s="17"/>
-      <c r="G3" s="17"/>
-      <c r="H3" s="17"/>
+      <c r="A3" s="28"/>
+      <c r="B3" s="28"/>
+      <c r="C3" s="28"/>
+      <c r="D3" s="28"/>
+      <c r="E3" s="28"/>
+      <c r="F3" s="28"/>
+      <c r="G3" s="28"/>
+      <c r="H3" s="28"/>
     </row>
     <row r="4" spans="1:8">
-      <c r="A4" s="18" t="s">
+      <c r="A4" s="29" t="s">
         <v>1</v>
       </c>
-      <c r="B4" s="17"/>
-      <c r="C4" s="19" t="s">
+      <c r="B4" s="28"/>
+      <c r="C4" s="30" t="s">
         <v>2</v>
       </c>
-      <c r="D4" s="17"/>
-      <c r="E4" s="17"/>
-      <c r="F4" s="17" t="s">
+      <c r="D4" s="28"/>
+      <c r="E4" s="28"/>
+      <c r="F4" s="28" t="s">
         <v>56</v>
       </c>
-      <c r="G4" s="17"/>
-      <c r="H4" s="17"/>
+      <c r="G4" s="28"/>
+      <c r="H4" s="28"/>
     </row>
     <row r="5" spans="1:8">
-      <c r="A5" s="17"/>
-      <c r="B5" s="17"/>
-      <c r="C5" s="17"/>
-      <c r="D5" s="17"/>
-      <c r="E5" s="17"/>
-      <c r="F5" s="17"/>
-      <c r="G5" s="17"/>
-      <c r="H5" s="17"/>
-    </row>
-    <row r="6" spans="1:8" ht="18">
+      <c r="A5" s="28"/>
+      <c r="B5" s="28"/>
+      <c r="C5" s="28"/>
+      <c r="D5" s="28"/>
+      <c r="E5" s="28"/>
+      <c r="F5" s="28"/>
+      <c r="G5" s="28"/>
+      <c r="H5" s="28"/>
+    </row>
+    <row r="6" spans="1:8" ht="18.75">
       <c r="A6" s="1" t="s">
         <v>4</v>
       </c>
@@ -2680,7 +3052,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="7" spans="1:8" ht="128.4" customHeight="1">
+    <row r="7" spans="1:8" ht="128.44999999999999" customHeight="1">
       <c r="A7" s="7">
         <v>1</v>
       </c>
@@ -2728,7 +3100,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="9" spans="1:8" ht="88.8" customHeight="1">
+    <row r="9" spans="1:8" ht="88.9" customHeight="1">
       <c r="A9" s="7">
         <v>3</v>
       </c>
@@ -2752,7 +3124,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="10" spans="1:8" ht="109.8" customHeight="1">
+    <row r="10" spans="1:8" ht="109.9" customHeight="1">
       <c r="A10" s="7">
         <v>4</v>
       </c>
@@ -2776,7 +3148,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="11" spans="1:8" ht="18">
+    <row r="11" spans="1:8" ht="18.75">
       <c r="A11" s="7">
         <v>5</v>
       </c>
@@ -2800,7 +3172,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="12" spans="1:8" ht="36">
+    <row r="12" spans="1:8" ht="37.5">
       <c r="A12" s="7">
         <v>6</v>
       </c>
@@ -2813,7 +3185,7 @@
       <c r="D12" s="7" t="s">
         <v>100</v>
       </c>
-      <c r="E12" s="20" t="s">
+      <c r="E12" s="14" t="s">
         <v>101</v>
       </c>
       <c r="F12" s="7"/>
@@ -2824,7 +3196,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="13" spans="1:8" ht="18">
+    <row r="13" spans="1:8" ht="37.5">
       <c r="A13" s="7">
         <v>7</v>
       </c>
@@ -2848,7 +3220,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="14" spans="1:8" ht="36">
+    <row r="14" spans="1:8" ht="37.5">
       <c r="A14" s="7">
         <v>8</v>
       </c>
@@ -2872,7 +3244,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="15" spans="1:8" ht="36">
+    <row r="15" spans="1:8" ht="37.5">
       <c r="A15" s="7">
         <v>9</v>
       </c>
@@ -2896,7 +3268,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="16" spans="1:8" ht="54">
+    <row r="16" spans="1:8" ht="56.25">
       <c r="A16" s="7">
         <v>10</v>
       </c>
@@ -2933,101 +3305,822 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:H6"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.4"/>
+  <dimension ref="A1:H42"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="16" customWidth="1"/>
-    <col min="2" max="2" width="18.109375" customWidth="1"/>
-    <col min="3" max="3" width="33.21875" customWidth="1"/>
-    <col min="4" max="5" width="21.21875" customWidth="1"/>
-    <col min="6" max="6" width="21.6640625" customWidth="1"/>
-    <col min="7" max="7" width="22.77734375" customWidth="1"/>
-    <col min="8" max="8" width="24.6640625" customWidth="1"/>
+    <col min="2" max="2" width="33.7109375" customWidth="1"/>
+    <col min="3" max="3" width="33.28515625" style="13" customWidth="1"/>
+    <col min="4" max="4" width="29" style="17" customWidth="1"/>
+    <col min="5" max="5" width="21.28515625" style="17" customWidth="1"/>
+    <col min="6" max="6" width="21.7109375" style="19" customWidth="1"/>
+    <col min="7" max="7" width="22.7109375" style="17" customWidth="1"/>
+    <col min="8" max="8" width="24.7109375" style="13" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:8">
-      <c r="A1" s="16" t="s">
+      <c r="A1" s="27" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="17"/>
-      <c r="C1" s="17"/>
-      <c r="D1" s="17"/>
-      <c r="E1" s="17"/>
-      <c r="F1" s="17"/>
-      <c r="G1" s="17"/>
-      <c r="H1" s="17"/>
+      <c r="B1" s="28"/>
+      <c r="C1" s="28"/>
+      <c r="D1" s="28"/>
+      <c r="E1" s="28"/>
+      <c r="F1" s="28"/>
+      <c r="G1" s="28"/>
+      <c r="H1" s="28"/>
     </row>
     <row r="2" spans="1:8">
-      <c r="A2" s="16"/>
-      <c r="B2" s="17"/>
-      <c r="C2" s="17"/>
-      <c r="D2" s="17"/>
-      <c r="E2" s="17"/>
-      <c r="F2" s="17"/>
-      <c r="G2" s="17"/>
-      <c r="H2" s="17"/>
+      <c r="A2" s="27"/>
+      <c r="B2" s="28"/>
+      <c r="C2" s="28"/>
+      <c r="D2" s="28"/>
+      <c r="E2" s="28"/>
+      <c r="F2" s="28"/>
+      <c r="G2" s="28"/>
+      <c r="H2" s="28"/>
     </row>
     <row r="3" spans="1:8">
-      <c r="A3" s="17"/>
-      <c r="B3" s="17"/>
-      <c r="C3" s="17"/>
-      <c r="D3" s="17"/>
-      <c r="E3" s="17"/>
-      <c r="F3" s="17"/>
-      <c r="G3" s="17"/>
-      <c r="H3" s="17"/>
+      <c r="A3" s="28"/>
+      <c r="B3" s="28"/>
+      <c r="C3" s="28"/>
+      <c r="D3" s="28"/>
+      <c r="E3" s="28"/>
+      <c r="F3" s="28"/>
+      <c r="G3" s="28"/>
+      <c r="H3" s="28"/>
     </row>
     <row r="4" spans="1:8">
-      <c r="A4" s="18" t="s">
+      <c r="A4" s="29" t="s">
         <v>1</v>
       </c>
-      <c r="B4" s="17"/>
-      <c r="C4" s="19" t="s">
+      <c r="B4" s="28"/>
+      <c r="C4" s="30" t="s">
         <v>2</v>
       </c>
-      <c r="D4" s="17"/>
-      <c r="E4" s="17"/>
-      <c r="F4" s="17" t="s">
+      <c r="D4" s="28"/>
+      <c r="E4" s="28"/>
+      <c r="F4" s="28" t="s">
         <v>58</v>
       </c>
-      <c r="G4" s="17"/>
-      <c r="H4" s="17"/>
+      <c r="G4" s="28"/>
+      <c r="H4" s="28"/>
     </row>
     <row r="5" spans="1:8">
-      <c r="A5" s="17"/>
-      <c r="B5" s="17"/>
-      <c r="C5" s="17"/>
-      <c r="D5" s="17"/>
-      <c r="E5" s="17"/>
-      <c r="F5" s="17"/>
-      <c r="G5" s="17"/>
-      <c r="H5" s="17"/>
-    </row>
-    <row r="6" spans="1:8" ht="18">
+      <c r="A5" s="28"/>
+      <c r="B5" s="28"/>
+      <c r="C5" s="28"/>
+      <c r="D5" s="28"/>
+      <c r="E5" s="28"/>
+      <c r="F5" s="28"/>
+      <c r="G5" s="28"/>
+      <c r="H5" s="28"/>
+    </row>
+    <row r="6" spans="1:8" ht="18.75">
       <c r="A6" s="1" t="s">
         <v>4</v>
       </c>
       <c r="B6" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="C6" s="1" t="s">
+      <c r="C6" s="15" t="s">
         <v>6</v>
       </c>
-      <c r="D6" s="1" t="s">
+      <c r="D6" s="16" t="s">
         <v>7</v>
       </c>
-      <c r="E6" s="1" t="s">
+      <c r="E6" s="16" t="s">
         <v>8</v>
       </c>
-      <c r="F6" s="1" t="s">
+      <c r="F6" s="18" t="s">
         <v>9</v>
       </c>
-      <c r="G6" s="1" t="s">
+      <c r="G6" s="16" t="s">
         <v>59</v>
       </c>
-      <c r="H6" s="1" t="s">
-        <v>60</v>
-      </c>
+      <c r="H6" s="15" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" s="20" customFormat="1" ht="132.75" customHeight="1">
+      <c r="A7" s="20">
+        <v>1</v>
+      </c>
+      <c r="B7" s="20" t="s">
+        <v>119</v>
+      </c>
+      <c r="C7" s="12" t="s">
+        <v>120</v>
+      </c>
+      <c r="D7" s="21" t="s">
+        <v>121</v>
+      </c>
+      <c r="E7" s="21" t="s">
+        <v>122</v>
+      </c>
+      <c r="F7" s="22" t="s">
+        <v>123</v>
+      </c>
+      <c r="G7" s="21" t="s">
+        <v>116</v>
+      </c>
+      <c r="H7" s="12" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" s="20" customFormat="1" ht="99" customHeight="1">
+      <c r="A8" s="20">
+        <v>2</v>
+      </c>
+      <c r="B8" s="20" t="s">
+        <v>119</v>
+      </c>
+      <c r="C8" s="12" t="s">
+        <v>120</v>
+      </c>
+      <c r="D8" s="21" t="s">
+        <v>124</v>
+      </c>
+      <c r="E8" s="21" t="s">
+        <v>125</v>
+      </c>
+      <c r="F8" s="22" t="s">
+        <v>126</v>
+      </c>
+      <c r="G8" s="21" t="s">
+        <v>116</v>
+      </c>
+      <c r="H8" s="12" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" s="20" customFormat="1" ht="99" customHeight="1">
+      <c r="A9" s="20">
+        <v>3</v>
+      </c>
+      <c r="B9" s="20" t="s">
+        <v>119</v>
+      </c>
+      <c r="C9" s="12" t="s">
+        <v>120</v>
+      </c>
+      <c r="D9" s="21" t="s">
+        <v>127</v>
+      </c>
+      <c r="E9" s="21" t="s">
+        <v>128</v>
+      </c>
+      <c r="F9" s="22" t="s">
+        <v>129</v>
+      </c>
+      <c r="G9" s="21" t="s">
+        <v>116</v>
+      </c>
+      <c r="H9" s="12" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" s="20" customFormat="1" ht="99" customHeight="1">
+      <c r="A10" s="20">
+        <v>4</v>
+      </c>
+      <c r="B10" s="20" t="s">
+        <v>119</v>
+      </c>
+      <c r="C10" s="12" t="s">
+        <v>120</v>
+      </c>
+      <c r="D10" s="21" t="s">
+        <v>130</v>
+      </c>
+      <c r="E10" s="21" t="s">
+        <v>131</v>
+      </c>
+      <c r="F10" s="22" t="s">
+        <v>132</v>
+      </c>
+      <c r="G10" s="21" t="s">
+        <v>116</v>
+      </c>
+      <c r="H10" s="12" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8" s="20" customFormat="1" ht="99" customHeight="1">
+      <c r="A11" s="20">
+        <v>5</v>
+      </c>
+      <c r="B11" s="20" t="s">
+        <v>119</v>
+      </c>
+      <c r="C11" s="12" t="s">
+        <v>120</v>
+      </c>
+      <c r="D11" s="21" t="s">
+        <v>133</v>
+      </c>
+      <c r="E11" s="21" t="s">
+        <v>134</v>
+      </c>
+      <c r="F11" s="22" t="s">
+        <v>135</v>
+      </c>
+      <c r="G11" s="21" t="s">
+        <v>116</v>
+      </c>
+      <c r="H11" s="12" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8" s="20" customFormat="1" ht="99" customHeight="1">
+      <c r="A12" s="20">
+        <v>6</v>
+      </c>
+      <c r="B12" s="20" t="s">
+        <v>119</v>
+      </c>
+      <c r="C12" s="12" t="s">
+        <v>120</v>
+      </c>
+      <c r="D12" s="21" t="s">
+        <v>136</v>
+      </c>
+      <c r="E12" s="21" t="s">
+        <v>137</v>
+      </c>
+      <c r="F12" s="22" t="s">
+        <v>138</v>
+      </c>
+      <c r="G12" s="21" t="s">
+        <v>116</v>
+      </c>
+      <c r="H12" s="12" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8" s="20" customFormat="1" ht="99" customHeight="1">
+      <c r="A13" s="20">
+        <v>7</v>
+      </c>
+      <c r="B13" s="20" t="s">
+        <v>119</v>
+      </c>
+      <c r="C13" s="12" t="s">
+        <v>120</v>
+      </c>
+      <c r="D13" s="21" t="s">
+        <v>139</v>
+      </c>
+      <c r="E13" s="21" t="s">
+        <v>140</v>
+      </c>
+      <c r="F13" s="22" t="s">
+        <v>141</v>
+      </c>
+      <c r="G13" s="21" t="s">
+        <v>116</v>
+      </c>
+      <c r="H13" s="12" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="14" spans="1:8" s="20" customFormat="1" ht="99" customHeight="1">
+      <c r="A14" s="20">
+        <v>8</v>
+      </c>
+      <c r="B14" s="20" t="s">
+        <v>119</v>
+      </c>
+      <c r="C14" s="12" t="s">
+        <v>120</v>
+      </c>
+      <c r="D14" s="21" t="s">
+        <v>142</v>
+      </c>
+      <c r="E14" s="21" t="s">
+        <v>143</v>
+      </c>
+      <c r="F14" s="22" t="s">
+        <v>144</v>
+      </c>
+      <c r="G14" s="21" t="s">
+        <v>116</v>
+      </c>
+      <c r="H14" s="12" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="15" spans="1:8" s="20" customFormat="1" ht="99" customHeight="1">
+      <c r="A15" s="20">
+        <v>9</v>
+      </c>
+      <c r="B15" s="20" t="s">
+        <v>119</v>
+      </c>
+      <c r="C15" s="12" t="s">
+        <v>120</v>
+      </c>
+      <c r="D15" s="21" t="s">
+        <v>145</v>
+      </c>
+      <c r="E15" s="21" t="s">
+        <v>146</v>
+      </c>
+      <c r="F15" s="22" t="s">
+        <v>147</v>
+      </c>
+      <c r="G15" s="21" t="s">
+        <v>116</v>
+      </c>
+      <c r="H15" s="12" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="16" spans="1:8" s="20" customFormat="1" ht="99" customHeight="1">
+      <c r="A16" s="20">
+        <v>10</v>
+      </c>
+      <c r="B16" s="20" t="s">
+        <v>119</v>
+      </c>
+      <c r="C16" s="12" t="s">
+        <v>120</v>
+      </c>
+      <c r="D16" s="21" t="s">
+        <v>148</v>
+      </c>
+      <c r="E16" s="21" t="s">
+        <v>149</v>
+      </c>
+      <c r="F16" s="22" t="s">
+        <v>150</v>
+      </c>
+      <c r="G16" s="21" t="s">
+        <v>116</v>
+      </c>
+      <c r="H16" s="12" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="17" spans="1:8" s="20" customFormat="1" ht="99" customHeight="1">
+      <c r="A17" s="20">
+        <v>11</v>
+      </c>
+      <c r="B17" s="20" t="s">
+        <v>119</v>
+      </c>
+      <c r="C17" s="12" t="s">
+        <v>120</v>
+      </c>
+      <c r="D17" s="21" t="s">
+        <v>151</v>
+      </c>
+      <c r="E17" s="21" t="s">
+        <v>152</v>
+      </c>
+      <c r="F17" s="22" t="s">
+        <v>153</v>
+      </c>
+      <c r="G17" s="21" t="s">
+        <v>116</v>
+      </c>
+      <c r="H17" s="12" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="18" spans="1:8" s="20" customFormat="1" ht="99" customHeight="1">
+      <c r="A18" s="20">
+        <v>12</v>
+      </c>
+      <c r="B18" s="20" t="s">
+        <v>119</v>
+      </c>
+      <c r="C18" s="12" t="s">
+        <v>120</v>
+      </c>
+      <c r="D18" s="21" t="s">
+        <v>154</v>
+      </c>
+      <c r="E18" s="21" t="s">
+        <v>155</v>
+      </c>
+      <c r="F18" s="22" t="s">
+        <v>156</v>
+      </c>
+      <c r="G18" s="21" t="s">
+        <v>116</v>
+      </c>
+      <c r="H18" s="12" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="19" spans="1:8" s="20" customFormat="1" ht="99" customHeight="1">
+      <c r="A19" s="20">
+        <v>13</v>
+      </c>
+      <c r="B19" s="20" t="s">
+        <v>119</v>
+      </c>
+      <c r="C19" s="12" t="s">
+        <v>120</v>
+      </c>
+      <c r="D19" s="21" t="s">
+        <v>157</v>
+      </c>
+      <c r="E19" s="21" t="s">
+        <v>158</v>
+      </c>
+      <c r="F19" s="22" t="s">
+        <v>159</v>
+      </c>
+      <c r="G19" s="21" t="s">
+        <v>116</v>
+      </c>
+      <c r="H19" s="12" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="20" spans="1:8" s="20" customFormat="1" ht="99" customHeight="1">
+      <c r="A20" s="20">
+        <v>14</v>
+      </c>
+      <c r="B20" s="20" t="s">
+        <v>119</v>
+      </c>
+      <c r="C20" s="12" t="s">
+        <v>120</v>
+      </c>
+      <c r="D20" s="21" t="s">
+        <v>160</v>
+      </c>
+      <c r="E20" s="21" t="s">
+        <v>161</v>
+      </c>
+      <c r="F20" s="22" t="s">
+        <v>162</v>
+      </c>
+      <c r="G20" s="21" t="s">
+        <v>116</v>
+      </c>
+      <c r="H20" s="12" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="21" spans="1:8" s="20" customFormat="1" ht="99" customHeight="1">
+      <c r="A21" s="20">
+        <v>15</v>
+      </c>
+      <c r="B21" s="20" t="s">
+        <v>119</v>
+      </c>
+      <c r="C21" s="12" t="s">
+        <v>120</v>
+      </c>
+      <c r="D21" s="21" t="s">
+        <v>163</v>
+      </c>
+      <c r="E21" s="21" t="s">
+        <v>164</v>
+      </c>
+      <c r="F21" s="22" t="s">
+        <v>165</v>
+      </c>
+      <c r="G21" s="21" t="s">
+        <v>116</v>
+      </c>
+      <c r="H21" s="12" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="22" spans="1:8" s="20" customFormat="1" ht="99" customHeight="1">
+      <c r="A22" s="20">
+        <v>16</v>
+      </c>
+      <c r="B22" s="20" t="s">
+        <v>166</v>
+      </c>
+      <c r="C22" s="12" t="s">
+        <v>120</v>
+      </c>
+      <c r="D22" s="21" t="s">
+        <v>167</v>
+      </c>
+      <c r="E22" s="21" t="s">
+        <v>168</v>
+      </c>
+      <c r="F22" s="22" t="s">
+        <v>169</v>
+      </c>
+      <c r="G22" s="21" t="s">
+        <v>116</v>
+      </c>
+      <c r="H22" s="12" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="23" spans="1:8" s="20" customFormat="1" ht="99" customHeight="1">
+      <c r="A23" s="20">
+        <v>17</v>
+      </c>
+      <c r="B23" s="20" t="s">
+        <v>166</v>
+      </c>
+      <c r="C23" s="12" t="s">
+        <v>120</v>
+      </c>
+      <c r="D23" s="21" t="s">
+        <v>170</v>
+      </c>
+      <c r="E23" s="21" t="s">
+        <v>171</v>
+      </c>
+      <c r="F23" s="22" t="s">
+        <v>172</v>
+      </c>
+      <c r="G23" s="21" t="s">
+        <v>116</v>
+      </c>
+      <c r="H23" s="12" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="24" spans="1:8" s="20" customFormat="1" ht="99" customHeight="1">
+      <c r="A24" s="20">
+        <v>18</v>
+      </c>
+      <c r="B24" s="20" t="s">
+        <v>166</v>
+      </c>
+      <c r="C24" s="12" t="s">
+        <v>120</v>
+      </c>
+      <c r="D24" s="21" t="s">
+        <v>173</v>
+      </c>
+      <c r="E24" s="21" t="s">
+        <v>174</v>
+      </c>
+      <c r="F24" s="22" t="s">
+        <v>175</v>
+      </c>
+      <c r="G24" s="21" t="s">
+        <v>116</v>
+      </c>
+      <c r="H24" s="12" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="25" spans="1:8" s="20" customFormat="1" ht="99" customHeight="1">
+      <c r="A25" s="20">
+        <v>19</v>
+      </c>
+      <c r="B25" s="20" t="s">
+        <v>166</v>
+      </c>
+      <c r="C25" s="12" t="s">
+        <v>120</v>
+      </c>
+      <c r="D25" s="21" t="s">
+        <v>176</v>
+      </c>
+      <c r="E25" s="21" t="s">
+        <v>177</v>
+      </c>
+      <c r="F25" s="22" t="s">
+        <v>178</v>
+      </c>
+      <c r="G25" s="21" t="s">
+        <v>116</v>
+      </c>
+      <c r="H25" s="12" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="26" spans="1:8" s="20" customFormat="1" ht="99" customHeight="1">
+      <c r="A26" s="20">
+        <v>20</v>
+      </c>
+      <c r="B26" s="20" t="s">
+        <v>166</v>
+      </c>
+      <c r="C26" s="12" t="s">
+        <v>120</v>
+      </c>
+      <c r="D26" s="21" t="s">
+        <v>179</v>
+      </c>
+      <c r="E26" s="21" t="s">
+        <v>180</v>
+      </c>
+      <c r="F26" s="22" t="s">
+        <v>181</v>
+      </c>
+      <c r="G26" s="21" t="s">
+        <v>116</v>
+      </c>
+      <c r="H26" s="12" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="27" spans="1:8" s="20" customFormat="1" ht="69" customHeight="1">
+      <c r="A27" s="20">
+        <v>21</v>
+      </c>
+      <c r="B27" s="20" t="s">
+        <v>166</v>
+      </c>
+      <c r="C27" s="12" t="s">
+        <v>120</v>
+      </c>
+      <c r="D27" s="21" t="s">
+        <v>182</v>
+      </c>
+      <c r="E27" s="21" t="s">
+        <v>183</v>
+      </c>
+      <c r="F27" s="22" t="s">
+        <v>184</v>
+      </c>
+      <c r="G27" s="21" t="s">
+        <v>116</v>
+      </c>
+      <c r="H27" s="12" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="28" spans="1:8" s="20" customFormat="1" ht="88.5" customHeight="1">
+      <c r="A28" s="20">
+        <v>22</v>
+      </c>
+      <c r="B28" s="20" t="s">
+        <v>166</v>
+      </c>
+      <c r="C28" s="12" t="s">
+        <v>120</v>
+      </c>
+      <c r="D28" s="21" t="s">
+        <v>185</v>
+      </c>
+      <c r="E28" s="21" t="s">
+        <v>186</v>
+      </c>
+      <c r="F28" s="22" t="s">
+        <v>187</v>
+      </c>
+      <c r="G28" s="21" t="s">
+        <v>116</v>
+      </c>
+      <c r="H28" s="12" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="29" spans="1:8" s="20" customFormat="1" ht="95.25" customHeight="1">
+      <c r="A29" s="20">
+        <v>23</v>
+      </c>
+      <c r="B29" s="20" t="s">
+        <v>166</v>
+      </c>
+      <c r="C29" s="12" t="s">
+        <v>120</v>
+      </c>
+      <c r="D29" s="21" t="s">
+        <v>188</v>
+      </c>
+      <c r="E29" s="21" t="s">
+        <v>189</v>
+      </c>
+      <c r="F29" s="22" t="s">
+        <v>190</v>
+      </c>
+      <c r="G29" s="21" t="s">
+        <v>116</v>
+      </c>
+      <c r="H29" s="12" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="30" spans="1:8" s="20" customFormat="1" ht="72.75" customHeight="1">
+      <c r="A30" s="20">
+        <v>24</v>
+      </c>
+      <c r="B30" s="20" t="s">
+        <v>191</v>
+      </c>
+      <c r="C30" s="12" t="s">
+        <v>120</v>
+      </c>
+      <c r="D30" s="21" t="s">
+        <v>192</v>
+      </c>
+      <c r="E30" s="21" t="s">
+        <v>193</v>
+      </c>
+      <c r="F30" s="22" t="s">
+        <v>194</v>
+      </c>
+      <c r="G30" s="21" t="s">
+        <v>116</v>
+      </c>
+      <c r="H30" s="12" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="31" spans="1:8" s="20" customFormat="1">
+      <c r="C31" s="12"/>
+      <c r="D31" s="21"/>
+      <c r="E31" s="21"/>
+      <c r="F31" s="22"/>
+      <c r="G31" s="21"/>
+      <c r="H31" s="12"/>
+    </row>
+    <row r="32" spans="1:8" s="20" customFormat="1">
+      <c r="C32" s="12"/>
+      <c r="D32" s="21"/>
+      <c r="E32" s="21"/>
+      <c r="F32" s="22"/>
+      <c r="G32" s="21"/>
+      <c r="H32" s="12"/>
+    </row>
+    <row r="33" spans="3:8" s="20" customFormat="1">
+      <c r="C33" s="12"/>
+      <c r="D33" s="21"/>
+      <c r="E33" s="21"/>
+      <c r="F33" s="22"/>
+      <c r="G33" s="21"/>
+      <c r="H33" s="12"/>
+    </row>
+    <row r="34" spans="3:8" s="20" customFormat="1">
+      <c r="C34" s="12"/>
+      <c r="D34" s="21"/>
+      <c r="E34" s="21"/>
+      <c r="F34" s="22"/>
+      <c r="G34" s="21"/>
+      <c r="H34" s="12"/>
+    </row>
+    <row r="35" spans="3:8" s="20" customFormat="1">
+      <c r="C35" s="12"/>
+      <c r="D35" s="21"/>
+      <c r="E35" s="21"/>
+      <c r="F35" s="22"/>
+      <c r="G35" s="21"/>
+      <c r="H35" s="12"/>
+    </row>
+    <row r="36" spans="3:8" s="20" customFormat="1">
+      <c r="C36" s="12"/>
+      <c r="D36" s="21"/>
+      <c r="E36" s="21"/>
+      <c r="F36" s="22"/>
+      <c r="G36" s="21"/>
+      <c r="H36" s="12"/>
+    </row>
+    <row r="37" spans="3:8" s="20" customFormat="1">
+      <c r="C37" s="12"/>
+      <c r="D37" s="21"/>
+      <c r="E37" s="21"/>
+      <c r="F37" s="22"/>
+      <c r="G37" s="21"/>
+      <c r="H37" s="12"/>
+    </row>
+    <row r="38" spans="3:8" s="20" customFormat="1">
+      <c r="C38" s="12"/>
+      <c r="D38" s="21"/>
+      <c r="E38" s="21"/>
+      <c r="F38" s="22"/>
+      <c r="G38" s="21"/>
+      <c r="H38" s="12"/>
+    </row>
+    <row r="39" spans="3:8" s="20" customFormat="1">
+      <c r="C39" s="12"/>
+      <c r="D39" s="21"/>
+      <c r="E39" s="21"/>
+      <c r="F39" s="22"/>
+      <c r="G39" s="21"/>
+      <c r="H39" s="12"/>
+    </row>
+    <row r="40" spans="3:8" s="20" customFormat="1">
+      <c r="C40" s="12"/>
+      <c r="D40" s="21"/>
+      <c r="E40" s="21"/>
+      <c r="F40" s="22"/>
+      <c r="G40" s="21"/>
+      <c r="H40" s="12"/>
+    </row>
+    <row r="41" spans="3:8" s="20" customFormat="1">
+      <c r="C41" s="12"/>
+      <c r="D41" s="21"/>
+      <c r="E41" s="21"/>
+      <c r="F41" s="22"/>
+      <c r="G41" s="21"/>
+      <c r="H41" s="12"/>
+    </row>
+    <row r="42" spans="3:8" s="20" customFormat="1">
+      <c r="C42" s="12"/>
+      <c r="D42" s="21"/>
+      <c r="E42" s="21"/>
+      <c r="F42" s="22"/>
+      <c r="G42" s="21"/>
+      <c r="H42" s="12"/>
     </row>
   </sheetData>
   <mergeCells count="4">
@@ -3043,77 +4136,77 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:H6"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="12.88671875" customWidth="1"/>
-    <col min="2" max="2" width="18.44140625" customWidth="1"/>
-    <col min="3" max="3" width="33.88671875" customWidth="1"/>
-    <col min="4" max="4" width="23.33203125" customWidth="1"/>
-    <col min="5" max="5" width="16.109375" customWidth="1"/>
-    <col min="6" max="6" width="25.109375" customWidth="1"/>
-    <col min="7" max="7" width="23.109375" customWidth="1"/>
-    <col min="8" max="8" width="27.77734375" customWidth="1"/>
+    <col min="1" max="1" width="12.85546875" customWidth="1"/>
+    <col min="2" max="2" width="18.42578125" customWidth="1"/>
+    <col min="3" max="3" width="33.85546875" customWidth="1"/>
+    <col min="4" max="4" width="23.28515625" customWidth="1"/>
+    <col min="5" max="5" width="16.140625" customWidth="1"/>
+    <col min="6" max="6" width="25.140625" customWidth="1"/>
+    <col min="7" max="7" width="23.140625" customWidth="1"/>
+    <col min="8" max="8" width="27.7109375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:8">
-      <c r="A1" s="16" t="s">
+      <c r="A1" s="27" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="17"/>
-      <c r="C1" s="17"/>
-      <c r="D1" s="17"/>
-      <c r="E1" s="17"/>
-      <c r="F1" s="17"/>
-      <c r="G1" s="17"/>
-      <c r="H1" s="17"/>
+      <c r="B1" s="28"/>
+      <c r="C1" s="28"/>
+      <c r="D1" s="28"/>
+      <c r="E1" s="28"/>
+      <c r="F1" s="28"/>
+      <c r="G1" s="28"/>
+      <c r="H1" s="28"/>
     </row>
     <row r="2" spans="1:8">
-      <c r="A2" s="16"/>
-      <c r="B2" s="17"/>
-      <c r="C2" s="17"/>
-      <c r="D2" s="17"/>
-      <c r="E2" s="17"/>
-      <c r="F2" s="17"/>
-      <c r="G2" s="17"/>
-      <c r="H2" s="17"/>
+      <c r="A2" s="27"/>
+      <c r="B2" s="28"/>
+      <c r="C2" s="28"/>
+      <c r="D2" s="28"/>
+      <c r="E2" s="28"/>
+      <c r="F2" s="28"/>
+      <c r="G2" s="28"/>
+      <c r="H2" s="28"/>
     </row>
     <row r="3" spans="1:8">
-      <c r="A3" s="17"/>
-      <c r="B3" s="17"/>
-      <c r="C3" s="17"/>
-      <c r="D3" s="17"/>
-      <c r="E3" s="17"/>
-      <c r="F3" s="17"/>
-      <c r="G3" s="17"/>
-      <c r="H3" s="17"/>
+      <c r="A3" s="28"/>
+      <c r="B3" s="28"/>
+      <c r="C3" s="28"/>
+      <c r="D3" s="28"/>
+      <c r="E3" s="28"/>
+      <c r="F3" s="28"/>
+      <c r="G3" s="28"/>
+      <c r="H3" s="28"/>
     </row>
     <row r="4" spans="1:8">
-      <c r="A4" s="18" t="s">
+      <c r="A4" s="29" t="s">
         <v>1</v>
       </c>
-      <c r="B4" s="17"/>
-      <c r="C4" s="19" t="s">
+      <c r="B4" s="28"/>
+      <c r="C4" s="30" t="s">
         <v>2</v>
       </c>
-      <c r="D4" s="17"/>
-      <c r="E4" s="17"/>
-      <c r="F4" s="17" t="s">
+      <c r="D4" s="28"/>
+      <c r="E4" s="28"/>
+      <c r="F4" s="28" t="s">
         <v>58</v>
       </c>
-      <c r="G4" s="17"/>
-      <c r="H4" s="17"/>
+      <c r="G4" s="28"/>
+      <c r="H4" s="28"/>
     </row>
     <row r="5" spans="1:8">
-      <c r="A5" s="17"/>
-      <c r="B5" s="17"/>
-      <c r="C5" s="17"/>
-      <c r="D5" s="17"/>
-      <c r="E5" s="17"/>
-      <c r="F5" s="17"/>
-      <c r="G5" s="17"/>
-      <c r="H5" s="17"/>
-    </row>
-    <row r="6" spans="1:8" ht="18">
+      <c r="A5" s="28"/>
+      <c r="B5" s="28"/>
+      <c r="C5" s="28"/>
+      <c r="D5" s="28"/>
+      <c r="E5" s="28"/>
+      <c r="F5" s="28"/>
+      <c r="G5" s="28"/>
+      <c r="H5" s="28"/>
+    </row>
+    <row r="6" spans="1:8" ht="18.75">
       <c r="A6" s="1" t="s">
         <v>4</v>
       </c>

</xml_diff>